<commit_message>
scan: seg0 2026-10-09 00:29 CST
</commit_message>
<xml_diff>
--- a/output/full_scan/batch_seq1_2026-10-08.xlsx
+++ b/output/full_scan/batch_seq1_2026-10-08.xlsx
@@ -552,10 +552,10 @@
         <v>0</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>80.17283677259813</v>
+        <v>80.17283677498976</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>30.21258045659086</v>
+        <v>30.21258054563315</v>
       </c>
       <c r="J2" s="2" t="n">
         <v>6.188783704430866</v>
@@ -570,7 +570,7 @@
         <v>-1</v>
       </c>
       <c r="N2" s="2" t="n">
-        <v>1.274804539708016</v>
+        <v>1.274804539808161</v>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
@@ -605,10 +605,10 @@
         <v>0</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>69.20121059785582</v>
+        <v>69.20121058570251</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>31.81656593284622</v>
+        <v>31.81656597158955</v>
       </c>
       <c r="J3" s="2" t="n">
         <v>2.784783857650602</v>
@@ -623,7 +623,7 @@
         <v>-1</v>
       </c>
       <c r="N3" s="2" t="n">
-        <v>0.7525762453040012</v>
+        <v>0.752576245493159</v>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
@@ -658,10 +658,10 @@
         <v>0</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>64.73263834905043</v>
+        <v>64.73263822920607</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>38.24791098672111</v>
+        <v>38.24791131681714</v>
       </c>
       <c r="J4" s="2" t="n">
         <v>2.665352528502424</v>
@@ -676,7 +676,7 @@
         <v>-1</v>
       </c>
       <c r="N4" s="2" t="n">
-        <v>4.460652700584408</v>
+        <v>4.460652702809876</v>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
@@ -711,10 +711,10 @@
         <v>0</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>70.89068027441786</v>
+        <v>70.8906803103731</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>27.31908780690902</v>
+        <v>27.3190878604013</v>
       </c>
       <c r="J5" s="2" t="n">
         <v>4.018966822028805</v>
@@ -729,7 +729,7 @@
         <v>-1</v>
       </c>
       <c r="N5" s="2" t="n">
-        <v>0.1328052751441823</v>
+        <v>0.1328052751330564</v>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
@@ -764,10 +764,10 @@
         <v>0</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>70.51754760136154</v>
+        <v>70.51754760490209</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>41.32971165203503</v>
+        <v>41.32971167159844</v>
       </c>
       <c r="J6" s="2" t="n">
         <v>2.469735452198493</v>
@@ -782,7 +782,7 @@
         <v>-1</v>
       </c>
       <c r="N6" s="2" t="n">
-        <v>0.1112840052726591</v>
+        <v>0.1112840052926858</v>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
@@ -817,10 +817,10 @@
         <v>0</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>64.87295561058221</v>
+        <v>64.87295581596869</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>31.78856377852052</v>
+        <v>31.7885638580313</v>
       </c>
       <c r="J7" s="2" t="n">
         <v>2.169258250102063</v>
@@ -835,7 +835,7 @@
         <v>-1</v>
       </c>
       <c r="N7" s="2" t="n">
-        <v>0.045136332984511</v>
+        <v>0.0451363329956377</v>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
@@ -856,7 +856,7 @@
         <v/>
       </c>
       <c r="D8" s="2" t="n">
-        <v>1040.908419774206</v>
+        <v>1040.908419774198</v>
       </c>
       <c r="E8" s="2" t="n">
         <v>26.95</v>
@@ -870,10 +870,10 @@
         <v>0</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>61.11680409464447</v>
+        <v>61.11680407478901</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>30.61470952734552</v>
+        <v>30.61470983579274</v>
       </c>
       <c r="J8" s="2" t="n">
         <v>3.517637716604867</v>
@@ -888,7 +888,7 @@
         <v>-1</v>
       </c>
       <c r="N8" s="2" t="n">
-        <v>0.0945599072711957</v>
+        <v>0.0945599074603575</v>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
@@ -923,10 +923,10 @@
         <v>0</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>63.69775655468641</v>
+        <v>63.69775659100706</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>23.0351335219685</v>
+        <v>23.0351335393537</v>
       </c>
       <c r="J9" s="2" t="n">
         <v>1.436548254733174</v>
@@ -941,7 +941,7 @@
         <v>-1</v>
       </c>
       <c r="N9" s="2" t="n">
-        <v>0.0135171220365246</v>
+        <v>0.0135171219475053</v>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
@@ -976,7 +976,7 @@
         <v>0</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>65.10548701378629</v>
+        <v>65.10548705143836</v>
       </c>
       <c r="I10" s="2" t="n">
         <v>16.38585827537656</v>
@@ -994,7 +994,7 @@
         <v>-1</v>
       </c>
       <c r="N10" s="2" t="n">
-        <v>0.08262516908424471</v>
+        <v>0.0826251691176256</v>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
@@ -1029,10 +1029,10 @@
         <v>0</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>60.1914546117352</v>
+        <v>60.19145462843796</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>41.95328179683475</v>
+        <v>41.95328184547853</v>
       </c>
       <c r="J11" s="2" t="n">
         <v>1.454658485441723</v>
@@ -1047,7 +1047,7 @@
         <v>-1</v>
       </c>
       <c r="N11" s="2" t="n">
-        <v>-0.0293590203718539</v>
+        <v>-0.0293590203607285</v>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
@@ -1068,7 +1068,7 @@
         <v/>
       </c>
       <c r="D12" s="2" t="n">
-        <v>986.4825838610114</v>
+        <v>986.482583861012</v>
       </c>
       <c r="E12" s="2" t="n">
         <v>13</v>
@@ -1082,10 +1082,10 @@
         <v>0</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>64.23333302659969</v>
+        <v>64.23333306825251</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>21.41760439273361</v>
+        <v>21.41760445922887</v>
       </c>
       <c r="J12" s="2" t="n">
         <v>2.010355149902084</v>
@@ -1100,7 +1100,7 @@
         <v>-1</v>
       </c>
       <c r="N12" s="2" t="n">
-        <v>0.0892334309966572</v>
+        <v>0.0892334310300391</v>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
@@ -1121,7 +1121,7 @@
         <v/>
       </c>
       <c r="D13" s="2" t="n">
-        <v>963.71328376913</v>
+        <v>963.7132837691298</v>
       </c>
       <c r="E13" s="2" t="n">
         <v>310</v>
@@ -1135,10 +1135,10 @@
         <v>0</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>76.71131973160895</v>
+        <v>76.71131973789321</v>
       </c>
       <c r="I13" s="2" t="n">
-        <v>38.78309003240684</v>
+        <v>38.78309007902674</v>
       </c>
       <c r="J13" s="2" t="n">
         <v>1.00909871808309</v>
@@ -1153,7 +1153,7 @@
         <v>-1</v>
       </c>
       <c r="N13" s="2" t="n">
-        <v>6.535923183604243</v>
+        <v>6.535923183871311</v>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
@@ -1188,10 +1188,10 @@
         <v>0</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>65.20017939670265</v>
+        <v>65.20017940538631</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>40.17082528149884</v>
+        <v>40.17082534131506</v>
       </c>
       <c r="J14" s="2" t="n">
         <v>1.086929629099419</v>
@@ -1206,7 +1206,7 @@
         <v>-1</v>
       </c>
       <c r="N14" s="2" t="n">
-        <v>0.0665875042217329</v>
+        <v>0.066587503992904</v>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
@@ -1241,10 +1241,10 @@
         <v>0</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>61.96836330729288</v>
+        <v>61.96836332775541</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>30.94990294516828</v>
+        <v>30.94990296910991</v>
       </c>
       <c r="J15" s="2" t="n">
         <v>2.157008870837585</v>
@@ -1259,7 +1259,7 @@
         <v>-1</v>
       </c>
       <c r="N15" s="2" t="n">
-        <v>0.0711981326298312</v>
+        <v>0.07119813266321259</v>
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
@@ -1294,10 +1294,10 @@
         <v>0</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>66.50573513352984</v>
+        <v>66.50573525073833</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>20.56815971474037</v>
+        <v>20.56815978218407</v>
       </c>
       <c r="J16" s="2" t="n">
         <v>3.133111364994963</v>
@@ -1312,7 +1312,7 @@
         <v>-1</v>
       </c>
       <c r="N16" s="2" t="n">
-        <v>0.0573879517725801</v>
+        <v>0.0573879517503264</v>
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
@@ -1347,10 +1347,10 @@
         <v>0</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>57.35964559474461</v>
+        <v>57.35964555180122</v>
       </c>
       <c r="I17" s="2" t="n">
-        <v>15.34434761927518</v>
+        <v>15.34434762138717</v>
       </c>
       <c r="J17" s="2" t="n">
         <v>1.080194659233564</v>
@@ -1400,10 +1400,10 @@
         <v>0</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>61.38298717825793</v>
+        <v>61.3829870749132</v>
       </c>
       <c r="I18" s="2" t="n">
-        <v>27.63174132414996</v>
+        <v>27.63174136957435</v>
       </c>
       <c r="J18" s="2" t="n">
         <v>1.186386890906387</v>
@@ -1418,7 +1418,7 @@
         <v>-1</v>
       </c>
       <c r="N18" s="2" t="n">
-        <v>2.052998328765589</v>
+        <v>2.052998328876865</v>
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
@@ -1453,10 +1453,10 @@
         <v>0</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>80.72403159768017</v>
+        <v>80.72403162355306</v>
       </c>
       <c r="I19" s="2" t="n">
-        <v>27.24659227592945</v>
+        <v>27.24659232732654</v>
       </c>
       <c r="J19" s="2" t="n">
         <v>7.946023953740562</v>
@@ -1471,7 +1471,7 @@
         <v>-1</v>
       </c>
       <c r="N19" s="2" t="n">
-        <v>0.4156284589936904</v>
+        <v>0.4156284589269245</v>
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
@@ -1506,10 +1506,10 @@
         <v>0</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>72.06372202939832</v>
+        <v>72.06372204378749</v>
       </c>
       <c r="I20" s="2" t="n">
-        <v>49.65411195735363</v>
+        <v>49.65411203780359</v>
       </c>
       <c r="J20" s="2" t="n">
         <v>0.2516352881706286</v>
@@ -1524,7 +1524,7 @@
         <v>-1</v>
       </c>
       <c r="N20" s="2" t="n">
-        <v>7.149312461256102</v>
+        <v>7.149312460588476</v>
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
@@ -1559,10 +1559,10 @@
         <v>0</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>74.21164350571729</v>
+        <v>74.21164350091702</v>
       </c>
       <c r="I21" s="2" t="n">
-        <v>62.99566184098345</v>
+        <v>62.99566189791751</v>
       </c>
       <c r="J21" s="2" t="n">
         <v>0.9414565960544968</v>
@@ -1577,7 +1577,7 @@
         <v>-1</v>
       </c>
       <c r="N21" s="2" t="n">
-        <v>0.8359666325601935</v>
+        <v>0.8359666324711732</v>
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
@@ -1612,10 +1612,10 @@
         <v>0</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>55.31063550903563</v>
+        <v>55.31063553190197</v>
       </c>
       <c r="I22" s="2" t="n">
-        <v>34.79945498266865</v>
+        <v>34.7994550079277</v>
       </c>
       <c r="J22" s="2" t="n">
         <v>1.203460007458598</v>
@@ -1630,7 +1630,7 @@
         <v>-1</v>
       </c>
       <c r="N22" s="2" t="n">
-        <v>0.022626734656678</v>
+        <v>0.022626734701186</v>
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
@@ -1665,10 +1665,10 @@
         <v>0</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>86.1273378843523</v>
+        <v>86.12733784641473</v>
       </c>
       <c r="I23" s="2" t="n">
-        <v>47.9582592599319</v>
+        <v>47.95825927001134</v>
       </c>
       <c r="J23" s="2" t="n">
         <v>2.478770809180932</v>
@@ -1718,10 +1718,10 @@
         <v>0</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>58.35918148471561</v>
+        <v>58.35918143127039</v>
       </c>
       <c r="I24" s="2" t="n">
-        <v>22.35063832092253</v>
+        <v>22.35063832506045</v>
       </c>
       <c r="J24" s="2" t="n">
         <v>0.8137865049238459</v>
@@ -1736,7 +1736,7 @@
         <v>-1</v>
       </c>
       <c r="N24" s="2" t="n">
-        <v>0.0308955017439934</v>
+        <v>0.0308955018107544</v>
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
@@ -1771,10 +1771,10 @@
         <v>0</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>60.78707800876577</v>
+        <v>60.78707803637715</v>
       </c>
       <c r="I25" s="2" t="n">
-        <v>41.19635166662874</v>
+        <v>41.19635168365246</v>
       </c>
       <c r="J25" s="2" t="n">
         <v>1.101693581738865</v>
@@ -1789,7 +1789,7 @@
         <v>-1</v>
       </c>
       <c r="N25" s="2" t="n">
-        <v>-0.0009089541805026</v>
+        <v>-0.0009089541716004</v>
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
@@ -1810,7 +1810,7 @@
         <v/>
       </c>
       <c r="D26" s="2" t="n">
-        <v>729.2300921619466</v>
+        <v>729.2300921619465</v>
       </c>
       <c r="E26" s="2" t="n">
         <v>17.95</v>
@@ -1824,10 +1824,10 @@
         <v>0</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>53.56031813780179</v>
+        <v>53.5603180470249</v>
       </c>
       <c r="I26" s="2" t="n">
-        <v>23.68266728059561</v>
+        <v>23.68266746806872</v>
       </c>
       <c r="J26" s="2" t="n">
         <v>0.4614597553978389</v>
@@ -1842,7 +1842,7 @@
         <v>-1</v>
       </c>
       <c r="N26" s="2" t="n">
-        <v>0.1079635445456977</v>
+        <v>0.1079635446219778</v>
       </c>
       <c r="O26" s="2" t="inlineStr">
         <is>
@@ -1863,7 +1863,7 @@
         <v/>
       </c>
       <c r="D27" s="2" t="n">
-        <v>706.9453848837485</v>
+        <v>706.9453848837487</v>
       </c>
       <c r="E27" s="2" t="n">
         <v>25.8</v>
@@ -1880,7 +1880,7 @@
         <v>53.88024028272982</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>31.53509193675142</v>
+        <v>31.535091878016</v>
       </c>
       <c r="J27" s="2" t="n">
         <v>0.5260641077467636</v>
@@ -1895,7 +1895,7 @@
         <v>-1</v>
       </c>
       <c r="N27" s="2" t="n">
-        <v>0.0431057183494682</v>
+        <v>0.0431057183160886</v>
       </c>
       <c r="O27" s="2" t="inlineStr">
         <is>
@@ -1916,7 +1916,7 @@
         <v/>
       </c>
       <c r="D28" s="2" t="n">
-        <v>697.2854171379371</v>
+        <v>697.2854171379375</v>
       </c>
       <c r="E28" s="2" t="n">
         <v>167</v>
@@ -1930,10 +1930,10 @@
         <v>0</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>52.74449369453678</v>
+        <v>52.74449371447933</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>8.543380747205095</v>
+        <v>8.543380743916792</v>
       </c>
       <c r="J28" s="2" t="n">
         <v>0.8309668319414185</v>
@@ -1948,7 +1948,7 @@
         <v>-1</v>
       </c>
       <c r="N28" s="2" t="n">
-        <v>0.1117792670590512</v>
+        <v>0.1117792673928514</v>
       </c>
       <c r="O28" s="2" t="inlineStr">
         <is>
@@ -1983,10 +1983,10 @@
         <v>0</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>58.56917045195578</v>
+        <v>58.56917052687851</v>
       </c>
       <c r="I29" s="2" t="n">
-        <v>33.40026640387457</v>
+        <v>33.40026644958505</v>
       </c>
       <c r="J29" s="2" t="n">
         <v>1.092231304575591</v>
@@ -2001,7 +2001,7 @@
         <v>-1</v>
       </c>
       <c r="N29" s="2" t="n">
-        <v>0.046751231041598</v>
+        <v>0.0467512310527251</v>
       </c>
       <c r="O29" s="2" t="inlineStr">
         <is>
@@ -2036,10 +2036,10 @@
         <v>0</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>54.45660340607546</v>
+        <v>54.45660325701563</v>
       </c>
       <c r="I30" s="2" t="n">
-        <v>13.78446988850994</v>
+        <v>13.78446990000659</v>
       </c>
       <c r="J30" s="2" t="n">
         <v>1.077817835173378</v>
@@ -2054,7 +2054,7 @@
         <v>-1</v>
       </c>
       <c r="N30" s="2" t="n">
-        <v>0.1306838958171621</v>
+        <v>0.1306838959506828</v>
       </c>
       <c r="O30" s="2" t="inlineStr">
         <is>
@@ -2089,10 +2089,10 @@
         <v>0</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>58.40651279137903</v>
+        <v>58.40651283713011</v>
       </c>
       <c r="I31" s="2" t="n">
-        <v>39.62181537445015</v>
+        <v>39.62181534004888</v>
       </c>
       <c r="J31" s="2" t="n">
         <v>0.8969147358565098</v>
@@ -2107,7 +2107,7 @@
         <v>-1</v>
       </c>
       <c r="N31" s="2" t="n">
-        <v>0.0543106075483959</v>
+        <v>0.0543106075261421</v>
       </c>
       <c r="O31" s="2" t="inlineStr">
         <is>
@@ -2128,7 +2128,7 @@
         <v/>
       </c>
       <c r="D32" s="2" t="n">
-        <v>686.9023908853073</v>
+        <v>686.9023908853081</v>
       </c>
       <c r="E32" s="2" t="n">
         <v>71.7</v>
@@ -2142,7 +2142,7 @@
         <v>0</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>56.25975808910625</v>
+        <v>56.25975825916096</v>
       </c>
       <c r="I32" s="2" t="n">
         <v>15.98731785562862</v>
@@ -2160,7 +2160,7 @@
         <v>-1</v>
       </c>
       <c r="N32" s="2" t="n">
-        <v>0.3252857665770791</v>
+        <v>0.3252857665325743</v>
       </c>
       <c r="O32" s="2" t="inlineStr">
         <is>
@@ -2195,10 +2195,10 @@
         <v>0</v>
       </c>
       <c r="H33" s="2" t="n">
-        <v>56.62016980465881</v>
+        <v>56.6201698096582</v>
       </c>
       <c r="I33" s="2" t="n">
-        <v>31.85762139150256</v>
+        <v>31.85762139324562</v>
       </c>
       <c r="J33" s="2" t="n">
         <v>4.219483892167547</v>
@@ -2248,10 +2248,10 @@
         <v>0</v>
       </c>
       <c r="H34" s="2" t="n">
-        <v>55.7243152322925</v>
+        <v>55.72431513553103</v>
       </c>
       <c r="I34" s="2" t="n">
-        <v>8.516846095654694</v>
+        <v>8.516846101263933</v>
       </c>
       <c r="J34" s="2" t="n">
         <v>1.134325838571727</v>
@@ -2266,7 +2266,7 @@
         <v>-1</v>
       </c>
       <c r="N34" s="2" t="n">
-        <v>0.0001716167618966</v>
+        <v>0.0001716168286608</v>
       </c>
       <c r="O34" s="2" t="inlineStr">
         <is>
@@ -2287,7 +2287,7 @@
         <v/>
       </c>
       <c r="D35" s="2" t="n">
-        <v>664.8039400019211</v>
+        <v>664.8039400019213</v>
       </c>
       <c r="E35" s="2" t="n">
         <v>26.05</v>
@@ -2301,10 +2301,10 @@
         <v>0</v>
       </c>
       <c r="H35" s="2" t="n">
-        <v>61.14563566662042</v>
+        <v>61.1456356822364</v>
       </c>
       <c r="I35" s="2" t="n">
-        <v>19.8754508141452</v>
+        <v>19.87545071030605</v>
       </c>
       <c r="J35" s="2" t="n">
         <v>0.9964773310473706</v>
@@ -2319,7 +2319,7 @@
         <v>-1</v>
       </c>
       <c r="N35" s="2" t="n">
-        <v>0.174858875555381</v>
+        <v>0.1748588758780659</v>
       </c>
       <c r="O35" s="2" t="inlineStr">
         <is>
@@ -2354,7 +2354,7 @@
         <v>0</v>
       </c>
       <c r="H36" s="2" t="n">
-        <v>56.08314224012081</v>
+        <v>56.08314226584429</v>
       </c>
       <c r="I36" s="2" t="n">
         <v>15.88962155302476</v>
@@ -2372,7 +2372,7 @@
         <v>-1</v>
       </c>
       <c r="N36" s="2" t="n">
-        <v>-0.0029866939320875</v>
+        <v>-0.0029866939432168</v>
       </c>
       <c r="O36" s="2" t="inlineStr">
         <is>
@@ -2393,7 +2393,7 @@
         <v/>
       </c>
       <c r="D37" s="2" t="n">
-        <v>573.598739150801</v>
+        <v>573.5987391508008</v>
       </c>
       <c r="E37" s="2" t="n">
         <v>18.65</v>
@@ -2407,10 +2407,10 @@
         <v>0</v>
       </c>
       <c r="H37" s="2" t="n">
-        <v>62.36392667966812</v>
+        <v>62.36392639714726</v>
       </c>
       <c r="I37" s="2" t="n">
-        <v>35.6557403312571</v>
+        <v>35.65574021052848</v>
       </c>
       <c r="J37" s="2" t="n">
         <v>0.5176600408040768</v>
@@ -2425,7 +2425,7 @@
         <v>-1</v>
       </c>
       <c r="N37" s="2" t="n">
-        <v>0.0943121663039842</v>
+        <v>0.0943121665042737</v>
       </c>
       <c r="O37" s="2" t="inlineStr">
         <is>
@@ -2460,10 +2460,10 @@
         <v>0</v>
       </c>
       <c r="H38" s="2" t="n">
-        <v>56.31338563474598</v>
+        <v>56.31338572741889</v>
       </c>
       <c r="I38" s="2" t="n">
-        <v>37.18109048749282</v>
+        <v>37.18109046029698</v>
       </c>
       <c r="J38" s="2" t="n">
         <v>0.2343401662160509</v>
@@ -2478,7 +2478,7 @@
         <v>-1</v>
       </c>
       <c r="N38" s="2" t="n">
-        <v>0.0618683372956318</v>
+        <v>0.0618683372622511</v>
       </c>
       <c r="O38" s="2" t="inlineStr">
         <is>
@@ -2513,10 +2513,10 @@
         <v>0</v>
       </c>
       <c r="H39" s="2" t="n">
-        <v>47.37128771143671</v>
+        <v>47.37128773022167</v>
       </c>
       <c r="I39" s="2" t="n">
-        <v>37.23378491266055</v>
+        <v>37.23378493046936</v>
       </c>
       <c r="J39" s="2" t="n">
         <v>0.4176033749544254</v>
@@ -2531,7 +2531,7 @@
         <v>-1</v>
       </c>
       <c r="N39" s="2" t="n">
-        <v>-0.8541210194205529</v>
+        <v>-0.8541210191535056</v>
       </c>
       <c r="O39" s="2" t="inlineStr">
         <is>
@@ -2566,10 +2566,10 @@
         <v>0</v>
       </c>
       <c r="H40" s="2" t="n">
-        <v>58.87775288409015</v>
+        <v>58.87775263406078</v>
       </c>
       <c r="I40" s="2" t="n">
-        <v>19.48016247149276</v>
+        <v>19.4801625473852</v>
       </c>
       <c r="J40" s="2" t="n">
         <v>1.44946356748814</v>
@@ -2584,7 +2584,7 @@
         <v>-1</v>
       </c>
       <c r="N40" s="2" t="n">
-        <v>0.0545869840830319</v>
+        <v>0.0545869841164134</v>
       </c>
       <c r="O40" s="2" t="inlineStr">
         <is>
@@ -2619,10 +2619,10 @@
         <v>0</v>
       </c>
       <c r="H41" s="2" t="n">
-        <v>53.15757120316218</v>
+        <v>53.1575712220322</v>
       </c>
       <c r="I41" s="2" t="n">
-        <v>11.68767622097894</v>
+        <v>11.6876762182732</v>
       </c>
       <c r="J41" s="2" t="n">
         <v>0.556293488945834</v>
@@ -2637,7 +2637,7 @@
         <v>-1</v>
       </c>
       <c r="N41" s="2" t="n">
-        <v>0.0362735806269461</v>
+        <v>0.0362735806158178</v>
       </c>
       <c r="O41" s="2" t="inlineStr">
         <is>
@@ -2672,10 +2672,10 @@
         <v>0</v>
       </c>
       <c r="H42" s="2" t="n">
-        <v>52.65346399341673</v>
+        <v>52.65346415520652</v>
       </c>
       <c r="I42" s="2" t="n">
-        <v>37.46372391050299</v>
+        <v>37.46372394343865</v>
       </c>
       <c r="J42" s="2" t="n">
         <v>0.2010716673320789</v>
@@ -2690,7 +2690,7 @@
         <v>-1</v>
       </c>
       <c r="N42" s="2" t="n">
-        <v>-0.3110437947869882</v>
+        <v>-0.3110437947313542</v>
       </c>
       <c r="O42" s="2" t="inlineStr">
         <is>
@@ -2725,7 +2725,7 @@
         <v>0</v>
       </c>
       <c r="H43" s="2" t="n">
-        <v>56.55829441302738</v>
+        <v>56.55829453134284</v>
       </c>
       <c r="I43" s="2" t="n">
         <v>20.97914438166865</v>
@@ -2743,7 +2743,7 @@
         <v>-1</v>
       </c>
       <c r="N43" s="2" t="n">
-        <v>0.0284657122430874</v>
+        <v>0.0284657122319598</v>
       </c>
       <c r="O43" s="2" t="inlineStr">
         <is>
@@ -2778,10 +2778,10 @@
         <v>0</v>
       </c>
       <c r="H44" s="2" t="n">
-        <v>51.14189598382556</v>
+        <v>51.14189599676926</v>
       </c>
       <c r="I44" s="2" t="n">
-        <v>21.96475349984593</v>
+        <v>21.96475352209658</v>
       </c>
       <c r="J44" s="2" t="n">
         <v>1.783222894230914</v>
@@ -2796,7 +2796,7 @@
         <v>-1</v>
       </c>
       <c r="N44" s="2" t="n">
-        <v>-1.090145901589991</v>
+        <v>-1.0901459017569</v>
       </c>
       <c r="O44" s="2" t="inlineStr">
         <is>
@@ -2831,10 +2831,10 @@
         <v>0</v>
       </c>
       <c r="H45" s="2" t="n">
-        <v>39.11962931976893</v>
+        <v>39.1196293527881</v>
       </c>
       <c r="I45" s="2" t="n">
-        <v>27.07119762474648</v>
+        <v>27.07119763782859</v>
       </c>
       <c r="J45" s="2" t="n">
         <v>0.9335601920955612</v>
@@ -2849,7 +2849,7 @@
         <v>-1</v>
       </c>
       <c r="N45" s="2" t="n">
-        <v>-0.004995393135652</v>
+        <v>-0.0049953932691792</v>
       </c>
       <c r="O45" s="2" t="inlineStr">
         <is>
@@ -2884,10 +2884,10 @@
         <v>0</v>
       </c>
       <c r="H46" s="2" t="n">
-        <v>52.40347474456304</v>
+        <v>52.40347475732364</v>
       </c>
       <c r="I46" s="2" t="n">
-        <v>4.726421337834694</v>
+        <v>4.726421381427445</v>
       </c>
       <c r="J46" s="2" t="n">
         <v>1.443319884863796</v>
@@ -2902,7 +2902,7 @@
         <v>-1</v>
       </c>
       <c r="N46" s="2" t="n">
-        <v>0.031036430253203</v>
+        <v>0.0310364302309483</v>
       </c>
       <c r="O46" s="2" t="inlineStr">
         <is>
@@ -2937,10 +2937,10 @@
         <v>0</v>
       </c>
       <c r="H47" s="2" t="n">
-        <v>64.70140804274459</v>
+        <v>64.70140804958056</v>
       </c>
       <c r="I47" s="2" t="n">
-        <v>62.17497336796992</v>
+        <v>62.17497344573913</v>
       </c>
       <c r="J47" s="2" t="n">
         <v>0.6355803468523609</v>
@@ -2955,7 +2955,7 @@
         <v>-1</v>
       </c>
       <c r="N47" s="2" t="n">
-        <v>0.2138992901004779</v>
+        <v>0.2138992901195479</v>
       </c>
       <c r="O47" s="2" t="inlineStr">
         <is>
@@ -2990,10 +2990,10 @@
         <v>0</v>
       </c>
       <c r="H48" s="2" t="n">
-        <v>51.1027497151034</v>
+        <v>51.10274972091622</v>
       </c>
       <c r="I48" s="2" t="n">
-        <v>12.10792042691007</v>
+        <v>12.10792045513235</v>
       </c>
       <c r="J48" s="2" t="n">
         <v>0.6754374092350689</v>
@@ -3029,7 +3029,7 @@
         <v/>
       </c>
       <c r="D49" s="2" t="n">
-        <v>456.4642151136923</v>
+        <v>456.4642151136927</v>
       </c>
       <c r="E49" s="2" t="n">
         <v>9.1</v>
@@ -3043,10 +3043,10 @@
         <v>0</v>
       </c>
       <c r="H49" s="2" t="n">
-        <v>59.29428234291891</v>
+        <v>59.29428232067028</v>
       </c>
       <c r="I49" s="2" t="n">
-        <v>13.52922296417572</v>
+        <v>13.52922294901413</v>
       </c>
       <c r="J49" s="2" t="n">
         <v>0.244590014339721</v>
@@ -3061,7 +3061,7 @@
         <v>-1</v>
       </c>
       <c r="N49" s="2" t="n">
-        <v>0.775193010464396</v>
+        <v>0.7751930105089038</v>
       </c>
       <c r="O49" s="2" t="inlineStr">
         <is>
@@ -3096,10 +3096,10 @@
         <v>0</v>
       </c>
       <c r="H50" s="2" t="n">
-        <v>48.75497587768669</v>
+        <v>48.75497590505417</v>
       </c>
       <c r="I50" s="2" t="n">
-        <v>17.65773682443178</v>
+        <v>17.65773684976121</v>
       </c>
       <c r="J50" s="2" t="n">
         <v>0.9171836345490876</v>
@@ -3114,7 +3114,7 @@
         <v>-1</v>
       </c>
       <c r="N50" s="2" t="n">
-        <v>0.1737957924784586</v>
+        <v>0.1737957924339361</v>
       </c>
       <c r="O50" s="2" t="inlineStr">
         <is>
@@ -3149,7 +3149,7 @@
         <v>0</v>
       </c>
       <c r="H51" s="2" t="n">
-        <v>49.55989811917836</v>
+        <v>49.55989816423709</v>
       </c>
       <c r="I51" s="2" t="n">
         <v>14.82984346640293</v>
@@ -3167,7 +3167,7 @@
         <v>-1</v>
       </c>
       <c r="N51" s="2" t="n">
-        <v>0.0414281014475445</v>
+        <v>0.0414281014252889</v>
       </c>
       <c r="O51" s="2" t="inlineStr">
         <is>
@@ -3202,10 +3202,10 @@
         <v>0</v>
       </c>
       <c r="H52" s="2" t="n">
-        <v>52.481475117373</v>
+        <v>52.48147513693962</v>
       </c>
       <c r="I52" s="2" t="n">
-        <v>8.649900948062754</v>
+        <v>8.649900945101788</v>
       </c>
       <c r="J52" s="2" t="n">
         <v>0.4090731176431278</v>
@@ -3220,7 +3220,7 @@
         <v>-1</v>
       </c>
       <c r="N52" s="2" t="n">
-        <v>0.0218674791921937</v>
+        <v>0.0218674791365578</v>
       </c>
       <c r="O52" s="2" t="inlineStr">
         <is>
@@ -3255,10 +3255,10 @@
         <v>0</v>
       </c>
       <c r="H53" s="2" t="n">
-        <v>53.77245534224674</v>
+        <v>53.77245546858805</v>
       </c>
       <c r="I53" s="2" t="n">
-        <v>19.59757042893624</v>
+        <v>19.59757051352537</v>
       </c>
       <c r="J53" s="2" t="n">
         <v>0.7354925662724614</v>
@@ -3273,7 +3273,7 @@
         <v>-1</v>
       </c>
       <c r="N53" s="2" t="n">
-        <v>0.009033423350009499</v>
+        <v>0.0090334233611363</v>
       </c>
       <c r="O53" s="2" t="inlineStr">
         <is>
@@ -3294,7 +3294,7 @@
         <v/>
       </c>
       <c r="D54" s="2" t="n">
-        <v>395.7555989745424</v>
+        <v>395.7555989745435</v>
       </c>
       <c r="E54" s="2" t="n">
         <v>17.15</v>
@@ -3308,10 +3308,10 @@
         <v>0</v>
       </c>
       <c r="H54" s="2" t="n">
-        <v>52.50674136460151</v>
+        <v>52.50674126073569</v>
       </c>
       <c r="I54" s="2" t="n">
-        <v>18.11407922422849</v>
+        <v>18.11407924387222</v>
       </c>
       <c r="J54" s="2" t="n">
         <v>2.619096366842568</v>
@@ -3326,7 +3326,7 @@
         <v>-1</v>
       </c>
       <c r="N54" s="2" t="n">
-        <v>0.0134957593356457</v>
+        <v>0.0134957593245204</v>
       </c>
       <c r="O54" s="2" t="inlineStr">
         <is>
@@ -3361,10 +3361,10 @@
         <v>0</v>
       </c>
       <c r="H55" s="2" t="n">
-        <v>53.51103911356375</v>
+        <v>53.51103909936661</v>
       </c>
       <c r="I55" s="2" t="n">
-        <v>8.456234766244982</v>
+        <v>8.456234704761002</v>
       </c>
       <c r="J55" s="2" t="n">
         <v>0.5690058807924451</v>
@@ -3379,7 +3379,7 @@
         <v>-1</v>
       </c>
       <c r="N55" s="2" t="n">
-        <v>0.9405787504818046</v>
+        <v>0.9405787507265928</v>
       </c>
       <c r="O55" s="2" t="inlineStr">
         <is>
@@ -3400,7 +3400,7 @@
         <v/>
       </c>
       <c r="D56" s="2" t="n">
-        <v>389.5086574968053</v>
+        <v>389.5086574968054</v>
       </c>
       <c r="E56" s="2" t="n">
         <v>13.15</v>
@@ -3414,10 +3414,10 @@
         <v>0</v>
       </c>
       <c r="H56" s="2" t="n">
-        <v>50.20325732302059</v>
+        <v>50.20325719991721</v>
       </c>
       <c r="I56" s="2" t="n">
-        <v>25.4158992698577</v>
+        <v>25.41589931029747</v>
       </c>
       <c r="J56" s="2" t="n">
         <v>0.8476163592073097</v>
@@ -3432,7 +3432,7 @@
         <v>-1</v>
       </c>
       <c r="N56" s="2" t="n">
-        <v>0.0067909159879053</v>
+        <v>0.0067909159990324</v>
       </c>
       <c r="O56" s="2" t="inlineStr">
         <is>
@@ -3467,10 +3467,10 @@
         <v>0</v>
       </c>
       <c r="H57" s="2" t="n">
-        <v>54.63154484914253</v>
+        <v>54.63154497065917</v>
       </c>
       <c r="I57" s="2" t="n">
-        <v>16.82689283339741</v>
+        <v>16.82689286159843</v>
       </c>
       <c r="J57" s="2" t="n">
         <v>1.021403050383265</v>
@@ -3485,7 +3485,7 @@
         <v>-1</v>
       </c>
       <c r="N57" s="2" t="n">
-        <v>0.0195329587186178</v>
+        <v>0.0195329586852375</v>
       </c>
       <c r="O57" s="2" t="inlineStr">
         <is>
@@ -3520,10 +3520,10 @@
         <v>0</v>
       </c>
       <c r="H58" s="2" t="n">
-        <v>51.86277082715442</v>
+        <v>51.86276959606941</v>
       </c>
       <c r="I58" s="2" t="n">
-        <v>8.884628204692039</v>
+        <v>8.884628207476135</v>
       </c>
       <c r="J58" s="2" t="n">
         <v>0.2012828426504924</v>
@@ -3538,7 +3538,7 @@
         <v>-1</v>
       </c>
       <c r="N58" s="2" t="n">
-        <v>-0.009139085972298899</v>
+        <v>-0.009139085983431</v>
       </c>
       <c r="O58" s="2" t="inlineStr">
         <is>
@@ -3573,10 +3573,10 @@
         <v>0</v>
       </c>
       <c r="H59" s="2" t="n">
-        <v>55.38532501627513</v>
+        <v>55.38532481591836</v>
       </c>
       <c r="I59" s="2" t="n">
-        <v>12.63650286869593</v>
+        <v>12.63650291873043</v>
       </c>
       <c r="J59" s="2" t="n">
         <v>0.6892411045184866</v>
@@ -3591,7 +3591,7 @@
         <v>-1</v>
       </c>
       <c r="N59" s="2" t="n">
-        <v>0.0942736517467922</v>
+        <v>0.0942736518691895</v>
       </c>
       <c r="O59" s="2" t="inlineStr">
         <is>
@@ -3626,10 +3626,10 @@
         <v>0</v>
       </c>
       <c r="H60" s="2" t="n">
-        <v>57.7548009149773</v>
+        <v>57.75480088203863</v>
       </c>
       <c r="I60" s="2" t="n">
-        <v>27.25558878962824</v>
+        <v>27.25558867824815</v>
       </c>
       <c r="J60" s="2" t="n">
         <v>0.7881415578388656</v>
@@ -3679,10 +3679,10 @@
         <v>0</v>
       </c>
       <c r="H61" s="2" t="n">
-        <v>35.28327264782266</v>
+        <v>35.28327272252579</v>
       </c>
       <c r="I61" s="2" t="n">
-        <v>46.9257514728259</v>
+        <v>46.92575169544239</v>
       </c>
       <c r="J61" s="2" t="n">
         <v>0.3770570139760966</v>
@@ -3697,7 +3697,7 @@
         <v>-1</v>
       </c>
       <c r="N61" s="2" t="n">
-        <v>0.0347248429720883</v>
+        <v>0.0347248429943436</v>
       </c>
       <c r="O61" s="2" t="inlineStr">
         <is>
@@ -3732,10 +3732,10 @@
         <v>0</v>
       </c>
       <c r="H62" s="2" t="n">
-        <v>48.04021486442525</v>
+        <v>48.04021488424984</v>
       </c>
       <c r="I62" s="2" t="n">
-        <v>18.79509929522317</v>
+        <v>18.79509926542985</v>
       </c>
       <c r="J62" s="2" t="n">
         <v>1.622855482725268</v>
@@ -3785,10 +3785,10 @@
         <v>0</v>
       </c>
       <c r="H63" s="2" t="n">
-        <v>46.50061872707418</v>
+        <v>46.50061881716901</v>
       </c>
       <c r="I63" s="2" t="n">
-        <v>8.01644658532725</v>
+        <v>8.016446644399693</v>
       </c>
       <c r="J63" s="2" t="n">
         <v>0.7693891200315155</v>
@@ -3803,7 +3803,7 @@
         <v>-1</v>
       </c>
       <c r="N63" s="2" t="n">
-        <v>0.2246841623609063</v>
+        <v>0.2246841619158339</v>
       </c>
       <c r="O63" s="2" t="inlineStr">
         <is>
@@ -3838,10 +3838,10 @@
         <v>0</v>
       </c>
       <c r="H64" s="2" t="n">
-        <v>37.88640007721988</v>
+        <v>37.88640013293856</v>
       </c>
       <c r="I64" s="2" t="n">
-        <v>33.46620769648086</v>
+        <v>33.46620779888283</v>
       </c>
       <c r="J64" s="2" t="n">
         <v>0.9406473455607608</v>
@@ -3856,7 +3856,7 @@
         <v>-1</v>
       </c>
       <c r="N64" s="2" t="n">
-        <v>0.1364726271616558</v>
+        <v>0.1364726272729277</v>
       </c>
       <c r="O64" s="2" t="inlineStr">
         <is>
@@ -3891,10 +3891,10 @@
         <v>0</v>
       </c>
       <c r="H65" s="2" t="n">
-        <v>45.13722421544097</v>
+        <v>45.13722423387938</v>
       </c>
       <c r="I65" s="2" t="n">
-        <v>17.40993185826983</v>
+        <v>17.4099317759493</v>
       </c>
       <c r="J65" s="2" t="n">
         <v>1.411806936854226</v>
@@ -3909,7 +3909,7 @@
         <v>-1</v>
       </c>
       <c r="N65" s="2" t="n">
-        <v>-0.0341555730871326</v>
+        <v>-0.034155573131642</v>
       </c>
       <c r="O65" s="2" t="inlineStr">
         <is>
@@ -3944,10 +3944,10 @@
         <v>0</v>
       </c>
       <c r="H66" s="2" t="n">
-        <v>47.7228819005116</v>
+        <v>47.72288222040269</v>
       </c>
       <c r="I66" s="2" t="n">
-        <v>28.92035833774281</v>
+        <v>28.92035837314694</v>
       </c>
       <c r="J66" s="2" t="n">
         <v>1.403074169411461</v>
@@ -3997,10 +3997,10 @@
         <v>0</v>
       </c>
       <c r="H67" s="2" t="n">
-        <v>44.90296668043416</v>
+        <v>44.90296660626093</v>
       </c>
       <c r="I67" s="2" t="n">
-        <v>11.03991006123469</v>
+        <v>11.03991005741066</v>
       </c>
       <c r="J67" s="2" t="n">
         <v>0.6663400244064923</v>
@@ -4015,7 +4015,7 @@
         <v>-1</v>
       </c>
       <c r="N67" s="2" t="n">
-        <v>-0.0058516856771119</v>
+        <v>-0.0058516856593089</v>
       </c>
       <c r="O67" s="2" t="inlineStr">
         <is>
@@ -4050,10 +4050,10 @@
         <v>0</v>
       </c>
       <c r="H68" s="2" t="n">
-        <v>42.78579988415291</v>
+        <v>42.78579994017417</v>
       </c>
       <c r="I68" s="2" t="n">
-        <v>7.411525856270829</v>
+        <v>7.411525866662092</v>
       </c>
       <c r="J68" s="2" t="n">
         <v>1.64993533516396</v>
@@ -4068,7 +4068,7 @@
         <v>-1</v>
       </c>
       <c r="N68" s="2" t="n">
-        <v>-0.0004846928192922</v>
+        <v>-0.0004846928860557</v>
       </c>
       <c r="O68" s="2" t="inlineStr">
         <is>
@@ -4103,10 +4103,10 @@
         <v>0</v>
       </c>
       <c r="H69" s="2" t="n">
-        <v>41.71233610336542</v>
+        <v>41.71233596904722</v>
       </c>
       <c r="I69" s="2" t="n">
-        <v>15.84257613489488</v>
+        <v>15.84257611083498</v>
       </c>
       <c r="J69" s="2" t="n">
         <v>1.723688155693854</v>
@@ -4121,7 +4121,7 @@
         <v>-1</v>
       </c>
       <c r="N69" s="2" t="n">
-        <v>0.0062445727039912</v>
+        <v>0.0062445727262468</v>
       </c>
       <c r="O69" s="2" t="inlineStr">
         <is>
@@ -4156,10 +4156,10 @@
         <v>0</v>
       </c>
       <c r="H70" s="2" t="n">
-        <v>44.14488040636909</v>
+        <v>44.14488045828641</v>
       </c>
       <c r="I70" s="2" t="n">
-        <v>20.86074910291989</v>
+        <v>20.86074912367117</v>
       </c>
       <c r="J70" s="2" t="n">
         <v>0.7910018241300343</v>
@@ -4174,7 +4174,7 @@
         <v>-1</v>
       </c>
       <c r="N70" s="2" t="n">
-        <v>-0.0173560273281909</v>
+        <v>-0.0173560272057868</v>
       </c>
       <c r="O70" s="2" t="inlineStr">
         <is>
@@ -4209,10 +4209,10 @@
         <v>0</v>
       </c>
       <c r="H71" s="2" t="n">
-        <v>48.07630345433294</v>
+        <v>48.07630339490873</v>
       </c>
       <c r="I71" s="2" t="n">
-        <v>7.753288955254289</v>
+        <v>7.753289027694827</v>
       </c>
       <c r="J71" s="2" t="n">
         <v>0.6464284826334502</v>
@@ -4227,7 +4227,7 @@
         <v>-1</v>
       </c>
       <c r="N71" s="2" t="n">
-        <v>0.0069723960574651</v>
+        <v>0.0069723960797198</v>
       </c>
       <c r="O71" s="2" t="inlineStr">
         <is>
@@ -4262,7 +4262,7 @@
         <v>0</v>
       </c>
       <c r="H72" s="2" t="n">
-        <v>39.84511980478589</v>
+        <v>39.84511966442652</v>
       </c>
       <c r="I72" s="2" t="n">
         <v>23.42096220064119</v>
@@ -4315,10 +4315,10 @@
         <v>0</v>
       </c>
       <c r="H73" s="2" t="n">
-        <v>49.79633145528607</v>
+        <v>49.79633150191531</v>
       </c>
       <c r="I73" s="2" t="n">
-        <v>19.90882855720587</v>
+        <v>19.90882861141895</v>
       </c>
       <c r="J73" s="2" t="n">
         <v>0.5721402003297253</v>
@@ -4333,7 +4333,7 @@
         <v>-1</v>
       </c>
       <c r="N73" s="2" t="n">
-        <v>0.031285927380799</v>
+        <v>0.0312859273718974</v>
       </c>
       <c r="O73" s="2" t="inlineStr">
         <is>
@@ -4368,10 +4368,10 @@
         <v>0</v>
       </c>
       <c r="H74" s="2" t="n">
-        <v>44.15346281561959</v>
+        <v>44.15346261208874</v>
       </c>
       <c r="I74" s="2" t="n">
-        <v>11.68058248716289</v>
+        <v>11.68058247187292</v>
       </c>
       <c r="J74" s="2" t="n">
         <v>0.8141012996267535</v>
@@ -4386,7 +4386,7 @@
         <v>-1</v>
       </c>
       <c r="N74" s="2" t="n">
-        <v>0.0062291217652151</v>
+        <v>0.0062291216984505</v>
       </c>
       <c r="O74" s="2" t="inlineStr">
         <is>
@@ -4421,7 +4421,7 @@
         <v>0</v>
       </c>
       <c r="H75" s="2" t="n">
-        <v>50.19395682133059</v>
+        <v>50.19395687493842</v>
       </c>
       <c r="I75" s="2" t="n">
         <v>12.77439717355541</v>
@@ -4439,7 +4439,7 @@
         <v>-1</v>
       </c>
       <c r="N75" s="2" t="n">
-        <v>0.2006751465583587</v>
+        <v>0.2006751466696338</v>
       </c>
       <c r="O75" s="2" t="inlineStr">
         <is>
@@ -4474,10 +4474,10 @@
         <v>0</v>
       </c>
       <c r="H76" s="2" t="n">
-        <v>38.18794987619042</v>
+        <v>38.18794992498007</v>
       </c>
       <c r="I76" s="2" t="n">
-        <v>13.70238405630391</v>
+        <v>13.70238417726834</v>
       </c>
       <c r="J76" s="2" t="n">
         <v>0.2663787681529267</v>
@@ -4492,7 +4492,7 @@
         <v>-1</v>
       </c>
       <c r="N76" s="2" t="n">
-        <v>-0.1785192374220403</v>
+        <v>-0.1785192374331628</v>
       </c>
       <c r="O76" s="2" t="inlineStr">
         <is>
@@ -4513,7 +4513,7 @@
         <v/>
       </c>
       <c r="D77" s="2" t="n">
-        <v>294.1304970482883</v>
+        <v>294.1304970482884</v>
       </c>
       <c r="E77" s="2" t="n">
         <v>71.09999999999999</v>
@@ -4527,7 +4527,7 @@
         <v>0</v>
       </c>
       <c r="H77" s="2" t="n">
-        <v>46.31372193087969</v>
+        <v>46.31372200022329</v>
       </c>
       <c r="I77" s="2" t="n">
         <v>18.96537150629971</v>
@@ -4566,7 +4566,7 @@
         <v/>
       </c>
       <c r="D78" s="2" t="n">
-        <v>290.5806475911314</v>
+        <v>290.5806475911313</v>
       </c>
       <c r="E78" s="2" t="n">
         <v>59.1</v>
@@ -4580,10 +4580,10 @@
         <v>0</v>
       </c>
       <c r="H78" s="2" t="n">
-        <v>51.84233897005343</v>
+        <v>51.84233896740086</v>
       </c>
       <c r="I78" s="2" t="n">
-        <v>9.636600581930583</v>
+        <v>9.63660060987506</v>
       </c>
       <c r="J78" s="2" t="n">
         <v>0.3769122477709995</v>
@@ -4598,7 +4598,7 @@
         <v>-1</v>
       </c>
       <c r="N78" s="2" t="n">
-        <v>-0.6833467802618758</v>
+        <v>-0.6833467800170778</v>
       </c>
       <c r="O78" s="2" t="inlineStr">
         <is>
@@ -4619,7 +4619,7 @@
         <v/>
       </c>
       <c r="D79" s="2" t="n">
-        <v>277.2716068120664</v>
+        <v>277.2716068120668</v>
       </c>
       <c r="E79" s="2" t="n">
         <v>15</v>
@@ -4633,10 +4633,10 @@
         <v>0</v>
       </c>
       <c r="H79" s="2" t="n">
-        <v>48.42739893914973</v>
+        <v>48.42739885642819</v>
       </c>
       <c r="I79" s="2" t="n">
-        <v>11.17146778924948</v>
+        <v>11.17146774627873</v>
       </c>
       <c r="J79" s="2" t="n">
         <v>0.611627332270861</v>
@@ -4651,7 +4651,7 @@
         <v>-1</v>
       </c>
       <c r="N79" s="2" t="n">
-        <v>0.0070284142272445</v>
+        <v>0.0070284142383726</v>
       </c>
       <c r="O79" s="2" t="inlineStr">
         <is>
@@ -4686,10 +4686,10 @@
         <v>0</v>
       </c>
       <c r="H80" s="2" t="n">
-        <v>42.06165097234261</v>
+        <v>42.06165126115096</v>
       </c>
       <c r="I80" s="2" t="n">
-        <v>26.62447196817286</v>
+        <v>26.62447215558087</v>
       </c>
       <c r="J80" s="2" t="n">
         <v>0.9096830556558836</v>
@@ -4704,7 +4704,7 @@
         <v>-1</v>
       </c>
       <c r="N80" s="2" t="n">
-        <v>0.0165672799395447</v>
+        <v>0.0165672795946073</v>
       </c>
       <c r="O80" s="2" t="inlineStr">
         <is>
@@ -4742,7 +4742,7 @@
         <v>54.33099145935613</v>
       </c>
       <c r="I81" s="2" t="n">
-        <v>19.41644921331924</v>
+        <v>19.41644925304152</v>
       </c>
       <c r="J81" s="2" t="n">
         <v>0.2335526867460398</v>
@@ -4757,7 +4757,7 @@
         <v>-1</v>
       </c>
       <c r="N81" s="2" t="n">
-        <v>0.0059784922720035</v>
+        <v>0.0059784922608734</v>
       </c>
       <c r="O81" s="2" t="inlineStr">
         <is>
@@ -4792,10 +4792,10 @@
         <v>0</v>
       </c>
       <c r="H82" s="2" t="n">
-        <v>54.69233758358904</v>
+        <v>54.69233759732294</v>
       </c>
       <c r="I82" s="2" t="n">
-        <v>26.29736000948895</v>
+        <v>26.29736003015393</v>
       </c>
       <c r="J82" s="2" t="n">
         <v>0.5449433764223256</v>
@@ -4810,7 +4810,7 @@
         <v>-1</v>
       </c>
       <c r="N82" s="2" t="n">
-        <v>0.0117528906793699</v>
+        <v>0.0117528906571208</v>
       </c>
       <c r="O82" s="2" t="inlineStr">
         <is>
@@ -4845,10 +4845,10 @@
         <v>0</v>
       </c>
       <c r="H83" s="2" t="n">
-        <v>39.78775280445137</v>
+        <v>39.7877528390004</v>
       </c>
       <c r="I83" s="2" t="n">
-        <v>7.913383339408423</v>
+        <v>7.913383344729607</v>
       </c>
       <c r="J83" s="2" t="n">
         <v>0.4114168995914857</v>
@@ -4863,7 +4863,7 @@
         <v>-1</v>
       </c>
       <c r="N83" s="2" t="n">
-        <v>0.1719188770072115</v>
+        <v>0.1719188767846322</v>
       </c>
       <c r="O83" s="2" t="inlineStr">
         <is>
@@ -4884,7 +4884,7 @@
         <v/>
       </c>
       <c r="D84" s="2" t="n">
-        <v>263.6836338648602</v>
+        <v>263.6836338648596</v>
       </c>
       <c r="E84" s="2" t="n">
         <v>65.90000000000001</v>
@@ -4898,10 +4898,10 @@
         <v>0</v>
       </c>
       <c r="H84" s="2" t="n">
-        <v>48.92356579320918</v>
+        <v>48.92356581487263</v>
       </c>
       <c r="I84" s="2" t="n">
-        <v>10.29367996991179</v>
+        <v>10.29368007246539</v>
       </c>
       <c r="J84" s="2" t="n">
         <v>0.1707632648460736</v>
@@ -4916,7 +4916,7 @@
         <v>-1</v>
       </c>
       <c r="N84" s="2" t="n">
-        <v>-0.0308113154394751</v>
+        <v>-0.0308113153727075</v>
       </c>
       <c r="O84" s="2" t="inlineStr">
         <is>
@@ -4951,10 +4951,10 @@
         <v>0</v>
       </c>
       <c r="H85" s="2" t="n">
-        <v>41.2537362484634</v>
+        <v>41.25373602648107</v>
       </c>
       <c r="I85" s="2" t="n">
-        <v>7.022032978871314</v>
+        <v>7.022033058927831</v>
       </c>
       <c r="J85" s="2" t="n">
         <v>0.4968064003889845</v>
@@ -4969,7 +4969,7 @@
         <v>-1</v>
       </c>
       <c r="N85" s="2" t="n">
-        <v>0.0968778423907766</v>
+        <v>0.09687784268008599</v>
       </c>
       <c r="O85" s="2" t="inlineStr">
         <is>
@@ -5004,10 +5004,10 @@
         <v>0</v>
       </c>
       <c r="H86" s="2" t="n">
-        <v>42.56936197952398</v>
+        <v>42.56936199569149</v>
       </c>
       <c r="I86" s="2" t="n">
-        <v>22.82800628437894</v>
+        <v>22.82800635326961</v>
       </c>
       <c r="J86" s="2" t="n">
         <v>0.3666024587756725</v>
@@ -5022,7 +5022,7 @@
         <v>-1</v>
       </c>
       <c r="N86" s="2" t="n">
-        <v>-0.0294667746213459</v>
+        <v>-0.0294667746658545</v>
       </c>
       <c r="O86" s="2" t="inlineStr">
         <is>
@@ -5043,7 +5043,7 @@
         <v/>
       </c>
       <c r="D87" s="2" t="n">
-        <v>257.7244651239459</v>
+        <v>257.7244651239454</v>
       </c>
       <c r="E87" s="2" t="n">
         <v>18.95</v>
@@ -5057,10 +5057,10 @@
         <v>0</v>
       </c>
       <c r="H87" s="2" t="n">
-        <v>21.53347188602778</v>
+        <v>21.53347183793444</v>
       </c>
       <c r="I87" s="2" t="n">
-        <v>43.4179578475856</v>
+        <v>43.41795780019862</v>
       </c>
       <c r="J87" s="2" t="n">
         <v>0.9403330658260024</v>
@@ -5075,7 +5075,7 @@
         <v>-1</v>
       </c>
       <c r="N87" s="2" t="n">
-        <v>-0.0491254250654281</v>
+        <v>-0.0491254250876836</v>
       </c>
       <c r="O87" s="2" t="inlineStr">
         <is>
@@ -5096,7 +5096,7 @@
         <v/>
       </c>
       <c r="D88" s="2" t="n">
-        <v>255.5890561059635</v>
+        <v>255.5890561059634</v>
       </c>
       <c r="E88" s="2" t="n">
         <v>8.16</v>
@@ -5110,10 +5110,10 @@
         <v>0</v>
       </c>
       <c r="H88" s="2" t="n">
-        <v>51.69900275886339</v>
+        <v>51.69900279750748</v>
       </c>
       <c r="I88" s="2" t="n">
-        <v>19.50131410284253</v>
+        <v>19.50131410284254</v>
       </c>
       <c r="J88" s="2" t="n">
         <v>0.4152215415283971</v>
@@ -5128,7 +5128,7 @@
         <v>-1</v>
       </c>
       <c r="N88" s="2" t="n">
-        <v>0.0209995453548116</v>
+        <v>0.0209995453570373</v>
       </c>
       <c r="O88" s="2" t="inlineStr">
         <is>
@@ -5149,7 +5149,7 @@
         <v/>
       </c>
       <c r="D89" s="2" t="n">
-        <v>252.584944961369</v>
+        <v>252.5849449613688</v>
       </c>
       <c r="E89" s="2" t="n">
         <v>6.13</v>
@@ -5163,10 +5163,10 @@
         <v>0</v>
       </c>
       <c r="H89" s="2" t="n">
-        <v>31.83446715951057</v>
+        <v>31.83446723487533</v>
       </c>
       <c r="I89" s="2" t="n">
-        <v>26.55960088006671</v>
+        <v>26.55960084823173</v>
       </c>
       <c r="J89" s="2" t="n">
         <v>0.8111406691347445</v>
@@ -5181,7 +5181,7 @@
         <v>-1</v>
       </c>
       <c r="N89" s="2" t="n">
-        <v>-0.0058522949663412</v>
+        <v>-0.0058522949730176</v>
       </c>
       <c r="O89" s="2" t="inlineStr">
         <is>
@@ -5216,10 +5216,10 @@
         <v>0</v>
       </c>
       <c r="H90" s="2" t="n">
-        <v>51.02451731635102</v>
+        <v>51.02451736710853</v>
       </c>
       <c r="I90" s="2" t="n">
-        <v>19.70385395091117</v>
+        <v>19.70385398545727</v>
       </c>
       <c r="J90" s="2" t="n">
         <v>0.6935591421593238</v>
@@ -5234,7 +5234,7 @@
         <v>-1</v>
       </c>
       <c r="N90" s="2" t="n">
-        <v>0.0271378726054624</v>
+        <v>0.0271378726032373</v>
       </c>
       <c r="O90" s="2" t="inlineStr">
         <is>
@@ -5272,7 +5272,7 @@
         <v>37.82205192790969</v>
       </c>
       <c r="I91" s="2" t="n">
-        <v>25.28069605936377</v>
+        <v>25.28069595562538</v>
       </c>
       <c r="J91" s="2" t="n">
         <v>0.4769121216376146</v>
@@ -5308,7 +5308,7 @@
         <v/>
       </c>
       <c r="D92" s="2" t="n">
-        <v>239.2644748569421</v>
+        <v>239.2644748569422</v>
       </c>
       <c r="E92" s="2" t="n">
         <v>13.35</v>
@@ -5322,7 +5322,7 @@
         <v>0</v>
       </c>
       <c r="H92" s="2" t="n">
-        <v>41.58594597784431</v>
+        <v>41.5859457568159</v>
       </c>
       <c r="I92" s="2" t="n">
         <v>16.69252899243765</v>
@@ -5340,7 +5340,7 @@
         <v>-1</v>
       </c>
       <c r="N92" s="2" t="n">
-        <v>0.0045336953344736</v>
+        <v>0.0045336953456002</v>
       </c>
       <c r="O92" s="2" t="inlineStr">
         <is>
@@ -5375,10 +5375,10 @@
         <v>0</v>
       </c>
       <c r="H93" s="2" t="n">
-        <v>40.26937575338695</v>
+        <v>40.26937586414288</v>
       </c>
       <c r="I93" s="2" t="n">
-        <v>45.48544007403331</v>
+        <v>45.48544014622911</v>
       </c>
       <c r="J93" s="2" t="n">
         <v>0.2675615452417887</v>
@@ -5393,7 +5393,7 @@
         <v>-1</v>
       </c>
       <c r="N93" s="2" t="n">
-        <v>-0.0127954454787933</v>
+        <v>-0.0127954455121749</v>
       </c>
       <c r="O93" s="2" t="inlineStr">
         <is>
@@ -5428,10 +5428,10 @@
         <v>0</v>
       </c>
       <c r="H94" s="2" t="n">
-        <v>47.56715242415966</v>
+        <v>47.56717939118548</v>
       </c>
       <c r="I94" s="2" t="n">
-        <v>6.115321759112116</v>
+        <v>6.115329549111436</v>
       </c>
       <c r="J94" s="2" t="n">
         <v>1.717771848461686</v>
@@ -5446,7 +5446,7 @@
         <v>-1</v>
       </c>
       <c r="N94" s="2" t="n">
-        <v>0.0380619836220317</v>
+        <v>0.0380618816205615</v>
       </c>
       <c r="O94" s="2" t="inlineStr">
         <is>
@@ -5481,10 +5481,10 @@
         <v>0</v>
       </c>
       <c r="H95" s="2" t="n">
-        <v>39.62324754182961</v>
+        <v>39.62324749719949</v>
       </c>
       <c r="I95" s="2" t="n">
-        <v>21.08291417144421</v>
+        <v>21.08291409982261</v>
       </c>
       <c r="J95" s="2" t="n">
         <v>0.5611447521286851</v>
@@ -5520,7 +5520,7 @@
         <v/>
       </c>
       <c r="D96" s="2" t="n">
-        <v>230.6780511349563</v>
+        <v>230.6780511349564</v>
       </c>
       <c r="E96" s="2" t="n">
         <v>13.15</v>
@@ -5534,10 +5534,10 @@
         <v>0</v>
       </c>
       <c r="H96" s="2" t="n">
-        <v>32.92146135478031</v>
+        <v>32.92146106644796</v>
       </c>
       <c r="I96" s="2" t="n">
-        <v>42.59826357240916</v>
+        <v>42.59826370699576</v>
       </c>
       <c r="J96" s="2" t="n">
         <v>0.944552593612224</v>
@@ -5552,7 +5552,7 @@
         <v>-1</v>
       </c>
       <c r="N96" s="2" t="n">
-        <v>-0.0028039410004986</v>
+        <v>-0.0028039409671167</v>
       </c>
       <c r="O96" s="2" t="inlineStr">
         <is>
@@ -5587,10 +5587,10 @@
         <v>0</v>
       </c>
       <c r="H97" s="2" t="n">
-        <v>43.15772216500528</v>
+        <v>43.15772217697669</v>
       </c>
       <c r="I97" s="2" t="n">
-        <v>18.3124119826131</v>
+        <v>18.31241188487894</v>
       </c>
       <c r="J97" s="2" t="n">
         <v>1.01989671559516</v>
@@ -5605,7 +5605,7 @@
         <v>-1</v>
       </c>
       <c r="N97" s="2" t="n">
-        <v>0.08265460056293621</v>
+        <v>0.0826546005518126</v>
       </c>
       <c r="O97" s="2" t="inlineStr">
         <is>
@@ -5640,10 +5640,10 @@
         <v>0</v>
       </c>
       <c r="H98" s="2" t="n">
-        <v>48.00136661924837</v>
+        <v>48.00136697318046</v>
       </c>
       <c r="I98" s="2" t="n">
-        <v>19.37917182415637</v>
+        <v>19.3791718622256</v>
       </c>
       <c r="J98" s="2" t="n">
         <v>0.9105529642281216</v>
@@ -5658,7 +5658,7 @@
         <v>-1</v>
       </c>
       <c r="N98" s="2" t="n">
-        <v>-0.0142412687682113</v>
+        <v>-0.0142412689351186</v>
       </c>
       <c r="O98" s="2" t="inlineStr">
         <is>
@@ -5693,10 +5693,10 @@
         <v>0</v>
       </c>
       <c r="H99" s="2" t="n">
-        <v>44.05183902270343</v>
+        <v>44.0518392129383</v>
       </c>
       <c r="I99" s="2" t="n">
-        <v>22.55702014090324</v>
+        <v>22.55702016405188</v>
       </c>
       <c r="J99" s="2" t="n">
         <v>0.6635766342353668</v>
@@ -5711,7 +5711,7 @@
         <v>-1</v>
       </c>
       <c r="N99" s="2" t="n">
-        <v>0.0185583537895728</v>
+        <v>0.0185583537228106</v>
       </c>
       <c r="O99" s="2" t="inlineStr">
         <is>
@@ -5746,10 +5746,10 @@
         <v>0</v>
       </c>
       <c r="H100" s="2" t="n">
-        <v>47.51653748912316</v>
+        <v>47.51653757506811</v>
       </c>
       <c r="I100" s="2" t="n">
-        <v>13.48716468452938</v>
+        <v>13.48716471547379</v>
       </c>
       <c r="J100" s="2" t="n">
         <v>0.5194008906363088</v>
@@ -5764,7 +5764,7 @@
         <v>-1</v>
       </c>
       <c r="N100" s="2" t="n">
-        <v>0.009562002512058</v>
+        <v>0.009562002489806</v>
       </c>
       <c r="O100" s="2" t="inlineStr">
         <is>
@@ -5799,10 +5799,10 @@
         <v>0</v>
       </c>
       <c r="H101" s="2" t="n">
-        <v>43.96490846280317</v>
+        <v>43.96490844058936</v>
       </c>
       <c r="I101" s="2" t="n">
-        <v>11.75004499029126</v>
+        <v>11.75004499502716</v>
       </c>
       <c r="J101" s="2" t="n">
         <v>0.9764873410534992</v>
@@ -5817,7 +5817,7 @@
         <v>-1</v>
       </c>
       <c r="N101" s="2" t="n">
-        <v>-0.6040818297321815</v>
+        <v>-0.6040818310675444</v>
       </c>
       <c r="O101" s="2" t="inlineStr">
         <is>
@@ -5852,10 +5852,10 @@
         <v>0</v>
       </c>
       <c r="H102" s="2" t="n">
-        <v>43.04425557437212</v>
+        <v>43.0442555503309</v>
       </c>
       <c r="I102" s="2" t="n">
-        <v>22.38786701543892</v>
+        <v>22.38786703202732</v>
       </c>
       <c r="J102" s="2" t="n">
         <v>1.205213533985461</v>
@@ -5870,7 +5870,7 @@
         <v>-1</v>
       </c>
       <c r="N102" s="2" t="n">
-        <v>0.0267939333279125</v>
+        <v>0.0267939333167843</v>
       </c>
       <c r="O102" s="2" t="inlineStr">
         <is>
@@ -5905,10 +5905,10 @@
         <v>0</v>
       </c>
       <c r="H103" s="2" t="n">
-        <v>50.01092533090651</v>
+        <v>50.01092528761991</v>
       </c>
       <c r="I103" s="2" t="n">
-        <v>10.81645838627808</v>
+        <v>10.8164583549112</v>
       </c>
       <c r="J103" s="2" t="n">
         <v>0.5284863780947551</v>
@@ -5958,10 +5958,10 @@
         <v>0</v>
       </c>
       <c r="H104" s="2" t="n">
-        <v>37.0426400723288</v>
+        <v>37.04264004047345</v>
       </c>
       <c r="I104" s="2" t="n">
-        <v>8.431701761978481</v>
+        <v>8.431701713439995</v>
       </c>
       <c r="J104" s="2" t="n">
         <v>0.5694832965869826</v>
@@ -5976,7 +5976,7 @@
         <v>-1</v>
       </c>
       <c r="N104" s="2" t="n">
-        <v>-0.0639165361780023</v>
+        <v>-0.06391653611123919</v>
       </c>
       <c r="O104" s="2" t="inlineStr">
         <is>
@@ -5997,7 +5997,7 @@
         <v/>
       </c>
       <c r="D105" s="2" t="n">
-        <v>218.4003149853265</v>
+        <v>218.4003149853268</v>
       </c>
       <c r="E105" s="2" t="n">
         <v>26.65</v>
@@ -6011,7 +6011,7 @@
         <v>0</v>
       </c>
       <c r="H105" s="2" t="n">
-        <v>35.3373673619852</v>
+        <v>35.33736724989028</v>
       </c>
       <c r="I105" s="2" t="n">
         <v>31.64443103445068</v>
@@ -6064,10 +6064,10 @@
         <v>0</v>
       </c>
       <c r="H106" s="2" t="n">
-        <v>51.63874245446677</v>
+        <v>51.63874253437996</v>
       </c>
       <c r="I106" s="2" t="n">
-        <v>11.44358228436945</v>
+        <v>11.44358241263085</v>
       </c>
       <c r="J106" s="2" t="n">
         <v>0.5224568862172136</v>
@@ -6082,7 +6082,7 @@
         <v>-1</v>
       </c>
       <c r="N106" s="2" t="n">
-        <v>0.0070268846018715</v>
+        <v>0.007026884668629</v>
       </c>
       <c r="O106" s="2" t="inlineStr">
         <is>
@@ -6117,10 +6117,10 @@
         <v>0</v>
       </c>
       <c r="H107" s="2" t="n">
-        <v>51.1489746772438</v>
+        <v>51.14897467808292</v>
       </c>
       <c r="I107" s="2" t="n">
-        <v>8.11752091748844</v>
+        <v>8.117520906096145</v>
       </c>
       <c r="J107" s="2" t="n">
         <v>0.4576731690936288</v>
@@ -6135,7 +6135,7 @@
         <v>-1</v>
       </c>
       <c r="N107" s="2" t="n">
-        <v>0.3063898763466445</v>
+        <v>0.3063898763688966</v>
       </c>
       <c r="O107" s="2" t="inlineStr">
         <is>
@@ -6156,7 +6156,7 @@
         <v/>
       </c>
       <c r="D108" s="2" t="n">
-        <v>213.99367107651</v>
+        <v>213.9936710765099</v>
       </c>
       <c r="E108" s="2" t="n">
         <v>36</v>
@@ -6173,7 +6173,7 @@
         <v>43.36465236607601</v>
       </c>
       <c r="I108" s="2" t="n">
-        <v>15.39280374509031</v>
+        <v>15.39280364553908</v>
       </c>
       <c r="J108" s="2" t="n">
         <v>0.6149201002736044</v>
@@ -6188,7 +6188,7 @@
         <v>-1</v>
       </c>
       <c r="N108" s="2" t="n">
-        <v>0.0363664549440032</v>
+        <v>0.0363664547659723</v>
       </c>
       <c r="O108" s="2" t="inlineStr">
         <is>
@@ -6223,10 +6223,10 @@
         <v>0</v>
       </c>
       <c r="H109" s="2" t="n">
-        <v>36.35251939521135</v>
+        <v>36.35251928457846</v>
       </c>
       <c r="I109" s="2" t="n">
-        <v>17.29578060318954</v>
+        <v>17.29578066225756</v>
       </c>
       <c r="J109" s="2" t="n">
         <v>1.03227059362489</v>
@@ -6241,7 +6241,7 @@
         <v>-1</v>
       </c>
       <c r="N109" s="2" t="n">
-        <v>0.0009951437375306999</v>
+        <v>0.0009951437709121999</v>
       </c>
       <c r="O109" s="2" t="inlineStr">
         <is>
@@ -6262,7 +6262,7 @@
         <v/>
       </c>
       <c r="D110" s="2" t="n">
-        <v>202.4923153694324</v>
+        <v>202.4923153694325</v>
       </c>
       <c r="E110" s="2" t="n">
         <v>26.4</v>
@@ -6276,10 +6276,10 @@
         <v>0</v>
       </c>
       <c r="H110" s="2" t="n">
-        <v>48.7718343781804</v>
+        <v>48.77183447279603</v>
       </c>
       <c r="I110" s="2" t="n">
-        <v>18.4773942522304</v>
+        <v>18.47739421942235</v>
       </c>
       <c r="J110" s="2" t="n">
         <v>0.8452227454692681</v>
@@ -6294,7 +6294,7 @@
         <v>-1</v>
       </c>
       <c r="N110" s="2" t="n">
-        <v>0.06739685749154831</v>
+        <v>0.0673968573135123</v>
       </c>
       <c r="O110" s="2" t="inlineStr">
         <is>
@@ -6315,7 +6315,7 @@
         <v/>
       </c>
       <c r="D111" s="2" t="n">
-        <v>198.7871125349718</v>
+        <v>198.7871125349714</v>
       </c>
       <c r="E111" s="2" t="n">
         <v>9.880000000000001</v>
@@ -6329,10 +6329,10 @@
         <v>0</v>
       </c>
       <c r="H111" s="2" t="n">
-        <v>40.57251210396802</v>
+        <v>40.57251241790832</v>
       </c>
       <c r="I111" s="2" t="n">
-        <v>16.35628201529903</v>
+        <v>16.3562819693102</v>
       </c>
       <c r="J111" s="2" t="n">
         <v>2.622220555204992</v>
@@ -6347,7 +6347,7 @@
         <v>-1</v>
       </c>
       <c r="N111" s="2" t="n">
-        <v>-0.0063514598154632</v>
+        <v>-0.0063514598265908</v>
       </c>
       <c r="O111" s="2" t="inlineStr">
         <is>
@@ -6382,10 +6382,10 @@
         <v>0</v>
       </c>
       <c r="H112" s="2" t="n">
-        <v>44.31756869858277</v>
+        <v>44.31756886840401</v>
       </c>
       <c r="I112" s="2" t="n">
-        <v>18.86867272923774</v>
+        <v>18.8686727620981</v>
       </c>
       <c r="J112" s="2" t="n">
         <v>0.3914240282644893</v>
@@ -6400,7 +6400,7 @@
         <v>-1</v>
       </c>
       <c r="N112" s="2" t="n">
-        <v>0.0855026918708359</v>
+        <v>0.0855026918930889</v>
       </c>
       <c r="O112" s="2" t="inlineStr">
         <is>
@@ -6435,10 +6435,10 @@
         <v>0</v>
       </c>
       <c r="H113" s="2" t="n">
-        <v>37.2786386031345</v>
+        <v>37.27863863390674</v>
       </c>
       <c r="I113" s="2" t="n">
-        <v>6.185853544885506</v>
+        <v>6.185853532291535</v>
       </c>
       <c r="J113" s="2" t="n">
         <v>0.4990335227507368</v>
@@ -6453,7 +6453,7 @@
         <v>-1</v>
       </c>
       <c r="N113" s="2" t="n">
-        <v>0.0034298141221704</v>
+        <v>0.0034298141110432</v>
       </c>
       <c r="O113" s="2" t="inlineStr">
         <is>
@@ -6474,7 +6474,7 @@
         <v/>
       </c>
       <c r="D114" s="2" t="n">
-        <v>186.4722149998801</v>
+        <v>186.47221499988</v>
       </c>
       <c r="E114" s="2" t="n">
         <v>9.31</v>
@@ -6491,7 +6491,7 @@
         <v>41.19338205689747</v>
       </c>
       <c r="I114" s="2" t="n">
-        <v>11.04183565137359</v>
+        <v>11.04183603296263</v>
       </c>
       <c r="J114" s="2" t="n">
         <v>1.063968515593518</v>
@@ -6506,7 +6506,7 @@
         <v>-1</v>
       </c>
       <c r="N114" s="2" t="n">
-        <v>0.0030659955490908</v>
+        <v>0.0030659955713453</v>
       </c>
       <c r="O114" s="2" t="inlineStr">
         <is>
@@ -6527,7 +6527,7 @@
         <v/>
       </c>
       <c r="D115" s="2" t="n">
-        <v>183.6321501429317</v>
+        <v>183.632150142932</v>
       </c>
       <c r="E115" s="2" t="n">
         <v>14.3</v>
@@ -6541,10 +6541,10 @@
         <v>0</v>
       </c>
       <c r="H115" s="2" t="n">
-        <v>47.54451069791222</v>
+        <v>47.54451072648457</v>
       </c>
       <c r="I115" s="2" t="n">
-        <v>17.48516680914093</v>
+        <v>17.48516682565103</v>
       </c>
       <c r="J115" s="2" t="n">
         <v>0.9005954513582841</v>
@@ -6559,7 +6559,7 @@
         <v>-1</v>
       </c>
       <c r="N115" s="2" t="n">
-        <v>-0.021596621682315</v>
+        <v>-0.0215966216934441</v>
       </c>
       <c r="O115" s="2" t="inlineStr">
         <is>
@@ -6594,10 +6594,10 @@
         <v>0</v>
       </c>
       <c r="H116" s="2" t="n">
-        <v>39.96530428691154</v>
+        <v>39.96530431894045</v>
       </c>
       <c r="I116" s="2" t="n">
-        <v>14.01694151477608</v>
+        <v>14.01694166133939</v>
       </c>
       <c r="J116" s="2" t="n">
         <v>1.455911996214547</v>
@@ -6612,7 +6612,7 @@
         <v>-1</v>
       </c>
       <c r="N116" s="2" t="n">
-        <v>0.0570931494249837</v>
+        <v>0.0570931494027361</v>
       </c>
       <c r="O116" s="2" t="inlineStr">
         <is>
@@ -6647,10 +6647,10 @@
         <v>0</v>
       </c>
       <c r="H117" s="2" t="n">
-        <v>31.67443343544602</v>
+        <v>31.67443362932927</v>
       </c>
       <c r="I117" s="2" t="n">
-        <v>16.91842408088984</v>
+        <v>16.91842415794158</v>
       </c>
       <c r="J117" s="2" t="n">
         <v>0.8953143695025576</v>
@@ -6665,7 +6665,7 @@
         <v>-1</v>
       </c>
       <c r="N117" s="2" t="n">
-        <v>-0.0965361363414818</v>
+        <v>-0.0965361360076679</v>
       </c>
       <c r="O117" s="2" t="inlineStr">
         <is>
@@ -6686,7 +6686,7 @@
         <v/>
       </c>
       <c r="D118" s="2" t="n">
-        <v>172.3742163260075</v>
+        <v>172.3742163260074</v>
       </c>
       <c r="E118" s="2" t="n">
         <v>9.949999999999999</v>
@@ -6700,10 +6700,10 @@
         <v>0</v>
       </c>
       <c r="H118" s="2" t="n">
-        <v>51.32341637521164</v>
+        <v>51.32341664702017</v>
       </c>
       <c r="I118" s="2" t="n">
-        <v>15.03198958530096</v>
+        <v>15.031989538943</v>
       </c>
       <c r="J118" s="2" t="n">
         <v>0.8771430071380611</v>
@@ -6718,7 +6718,7 @@
         <v>-1</v>
       </c>
       <c r="N118" s="2" t="n">
-        <v>-0.0049623190408491</v>
+        <v>-0.0049623190631047</v>
       </c>
       <c r="O118" s="2" t="inlineStr">
         <is>
@@ -6739,7 +6739,7 @@
         <v/>
       </c>
       <c r="D119" s="2" t="n">
-        <v>172.2445233747418</v>
+        <v>172.2445233747422</v>
       </c>
       <c r="E119" s="2" t="n">
         <v>106.5</v>
@@ -6753,10 +6753,10 @@
         <v>0</v>
       </c>
       <c r="H119" s="2" t="n">
-        <v>48.99849346929168</v>
+        <v>48.99849359283251</v>
       </c>
       <c r="I119" s="2" t="n">
-        <v>13.91925366078436</v>
+        <v>13.91925374940691</v>
       </c>
       <c r="J119" s="2" t="n">
         <v>0.7911795727396692</v>
@@ -6771,7 +6771,7 @@
         <v>-1</v>
       </c>
       <c r="N119" s="2" t="n">
-        <v>-0.0139062412930579</v>
+        <v>-0.0139062409592394</v>
       </c>
       <c r="O119" s="2" t="inlineStr">
         <is>
@@ -6792,7 +6792,7 @@
         <v/>
       </c>
       <c r="D120" s="2" t="n">
-        <v>167.5457013370639</v>
+        <v>167.545701337064</v>
       </c>
       <c r="E120" s="2" t="n">
         <v>42.75</v>
@@ -6806,10 +6806,10 @@
         <v>0</v>
       </c>
       <c r="H120" s="2" t="n">
-        <v>44.49064374825022</v>
+        <v>44.4906437930235</v>
       </c>
       <c r="I120" s="2" t="n">
-        <v>9.890374470430356</v>
+        <v>9.890374513089109</v>
       </c>
       <c r="J120" s="2" t="n">
         <v>1.25653611940896</v>
@@ -6824,7 +6824,7 @@
         <v>-1</v>
       </c>
       <c r="N120" s="2" t="n">
-        <v>-0.0119185455109847</v>
+        <v>-0.0119185456445133</v>
       </c>
       <c r="O120" s="2" t="inlineStr">
         <is>
@@ -6859,10 +6859,10 @@
         <v>0</v>
       </c>
       <c r="H121" s="2" t="n">
-        <v>30.40707576683207</v>
+        <v>30.40707575332539</v>
       </c>
       <c r="I121" s="2" t="n">
-        <v>38.55859947648016</v>
+        <v>38.55859951359474</v>
       </c>
       <c r="J121" s="2" t="n">
         <v>0.311157353532924</v>
@@ -6877,7 +6877,7 @@
         <v>-1</v>
       </c>
       <c r="N121" s="2" t="n">
-        <v>-0.048529174648822</v>
+        <v>-0.0485291746599488</v>
       </c>
       <c r="O121" s="2" t="inlineStr">
         <is>
@@ -6912,10 +6912,10 @@
         <v>0</v>
       </c>
       <c r="H122" s="2" t="n">
-        <v>35.00249401108452</v>
+        <v>35.00249362280672</v>
       </c>
       <c r="I122" s="2" t="n">
-        <v>15.19103208076683</v>
+        <v>15.1910321276286</v>
       </c>
       <c r="J122" s="2" t="n">
         <v>1.237176790090185</v>
@@ -6930,7 +6930,7 @@
         <v>-1</v>
       </c>
       <c r="N122" s="2" t="n">
-        <v>-0.0173587360195369</v>
+        <v>-0.0173587358415028</v>
       </c>
       <c r="O122" s="2" t="inlineStr">
         <is>
@@ -6951,7 +6951,7 @@
         <v/>
       </c>
       <c r="D123" s="2" t="n">
-        <v>163.1587006581296</v>
+        <v>163.1587006581297</v>
       </c>
       <c r="E123" s="2" t="n">
         <v>6.27</v>
@@ -6965,10 +6965,10 @@
         <v>0</v>
       </c>
       <c r="H123" s="2" t="n">
-        <v>49.62774985998078</v>
+        <v>49.62774979660142</v>
       </c>
       <c r="I123" s="2" t="n">
-        <v>13.51074371859988</v>
+        <v>13.51074375135028</v>
       </c>
       <c r="J123" s="2" t="n">
         <v>0.6366568004194362</v>
@@ -6983,7 +6983,7 @@
         <v>-1</v>
       </c>
       <c r="N123" s="2" t="n">
-        <v>0.0280658943119384</v>
+        <v>0.0280658942830072</v>
       </c>
       <c r="O123" s="2" t="inlineStr">
         <is>
@@ -7018,10 +7018,10 @@
         <v>0</v>
       </c>
       <c r="H124" s="2" t="n">
-        <v>51.87251764236824</v>
+        <v>51.87251749724368</v>
       </c>
       <c r="I124" s="2" t="n">
-        <v>12.79069677105256</v>
+        <v>12.79069701805218</v>
       </c>
       <c r="J124" s="2" t="n">
         <v>0.3375353914095136</v>
@@ -7036,7 +7036,7 @@
         <v>-1</v>
       </c>
       <c r="N124" s="2" t="n">
-        <v>0.0822249490819298</v>
+        <v>0.08222494928221739</v>
       </c>
       <c r="O124" s="2" t="inlineStr">
         <is>
@@ -7057,7 +7057,7 @@
         <v/>
       </c>
       <c r="D125" s="2" t="n">
-        <v>155.7147432784421</v>
+        <v>155.7147432784423</v>
       </c>
       <c r="E125" s="2" t="n">
         <v>21.75</v>
@@ -7071,10 +7071,10 @@
         <v>0</v>
       </c>
       <c r="H125" s="2" t="n">
-        <v>35.15927503302262</v>
+        <v>35.15927462792179</v>
       </c>
       <c r="I125" s="2" t="n">
-        <v>20.48553242813232</v>
+        <v>20.48553256967309</v>
       </c>
       <c r="J125" s="2" t="n">
         <v>0.3005727525106256</v>
@@ -7089,7 +7089,7 @@
         <v>-1</v>
       </c>
       <c r="N125" s="2" t="n">
-        <v>-0.0822687416686408</v>
+        <v>-0.0822687415017324</v>
       </c>
       <c r="O125" s="2" t="inlineStr">
         <is>
@@ -7110,7 +7110,7 @@
         <v/>
       </c>
       <c r="D126" s="2" t="n">
-        <v>152.2473752386857</v>
+        <v>152.2473752386855</v>
       </c>
       <c r="E126" s="2" t="n">
         <v>26.2</v>
@@ -7124,10 +7124,10 @@
         <v>0</v>
       </c>
       <c r="H126" s="2" t="n">
-        <v>31.18159499542652</v>
+        <v>31.18159486352656</v>
       </c>
       <c r="I126" s="2" t="n">
-        <v>24.80112973990667</v>
+        <v>24.80112969310196</v>
       </c>
       <c r="J126" s="2" t="n">
         <v>1.025092085012192</v>
@@ -7142,7 +7142,7 @@
         <v>-1</v>
       </c>
       <c r="N126" s="2" t="n">
-        <v>-0.0117486480746502</v>
+        <v>-0.0117486480078891</v>
       </c>
       <c r="O126" s="2" t="inlineStr">
         <is>
@@ -7177,10 +7177,10 @@
         <v>0</v>
       </c>
       <c r="H127" s="2" t="n">
-        <v>47.39263027774812</v>
+        <v>47.39263037244685</v>
       </c>
       <c r="I127" s="2" t="n">
-        <v>8.566954855793488</v>
+        <v>8.566954861202273</v>
       </c>
       <c r="J127" s="2" t="n">
         <v>0.1845698724182319</v>
@@ -7195,7 +7195,7 @@
         <v>-1</v>
       </c>
       <c r="N127" s="2" t="n">
-        <v>0.0391163732702641</v>
+        <v>0.0391163732146318</v>
       </c>
       <c r="O127" s="2" t="inlineStr">
         <is>
@@ -7216,7 +7216,7 @@
         <v/>
       </c>
       <c r="D128" s="2" t="n">
-        <v>130.7674920088215</v>
+        <v>130.7674920088214</v>
       </c>
       <c r="E128" s="2" t="n">
         <v>20.5</v>
@@ -7230,10 +7230,10 @@
         <v>0</v>
       </c>
       <c r="H128" s="2" t="n">
-        <v>51.07066526029325</v>
+        <v>51.07066525747229</v>
       </c>
       <c r="I128" s="2" t="n">
-        <v>15.89755370173826</v>
+        <v>15.89755363583524</v>
       </c>
       <c r="J128" s="2" t="n">
         <v>0.6976466133949744</v>
@@ -7248,7 +7248,7 @@
         <v>-1</v>
       </c>
       <c r="N128" s="2" t="n">
-        <v>0.4654882144933212</v>
+        <v>0.4654882145155766</v>
       </c>
       <c r="O128" s="2" t="inlineStr">
         <is>
@@ -7283,10 +7283,10 @@
         <v>0</v>
       </c>
       <c r="H129" s="2" t="n">
-        <v>48.1318591633833</v>
+        <v>48.13185912848309</v>
       </c>
       <c r="I129" s="2" t="n">
-        <v>8.755288088478709</v>
+        <v>8.755288046658189</v>
       </c>
       <c r="J129" s="2" t="n">
         <v>1.101457677301412</v>
@@ -7322,7 +7322,7 @@
         <v/>
       </c>
       <c r="D130" s="2" t="n">
-        <v>114.5668906328587</v>
+        <v>114.5668906328588</v>
       </c>
       <c r="E130" s="2" t="n">
         <v>18.95</v>
@@ -7336,10 +7336,10 @@
         <v>0</v>
       </c>
       <c r="H130" s="2" t="n">
-        <v>37.95493196905961</v>
+        <v>37.95493209600016</v>
       </c>
       <c r="I130" s="2" t="n">
-        <v>10.84590886708707</v>
+        <v>10.84590893064599</v>
       </c>
       <c r="J130" s="2" t="n">
         <v>0.9647153596768696</v>
@@ -7354,7 +7354,7 @@
         <v>-1</v>
       </c>
       <c r="N130" s="2" t="n">
-        <v>-0.0371663844339656</v>
+        <v>-0.0371663844450914</v>
       </c>
       <c r="O130" s="2" t="inlineStr">
         <is>
@@ -7375,7 +7375,7 @@
         <v/>
       </c>
       <c r="D131" s="2" t="n">
-        <v>82.62113206728321</v>
+        <v>82.62113206728273</v>
       </c>
       <c r="E131" s="2" t="n">
         <v>63.2</v>
@@ -7389,10 +7389,10 @@
         <v>0</v>
       </c>
       <c r="H131" s="2" t="n">
-        <v>50.5378685570446</v>
+        <v>50.53786853606798</v>
       </c>
       <c r="I131" s="2" t="n">
-        <v>13.5747996949799</v>
+        <v>13.5747996254918</v>
       </c>
       <c r="J131" s="2" t="n">
         <v>0.792316615578036</v>
@@ -7407,7 +7407,7 @@
         <v>-1</v>
       </c>
       <c r="N131" s="2" t="n">
-        <v>0.851757224042538</v>
+        <v>0.8517572242428235</v>
       </c>
       <c r="O131" s="2" t="inlineStr">
         <is>
@@ -7445,7 +7445,7 @@
         <v>44.1707211614111</v>
       </c>
       <c r="I132" s="2" t="n">
-        <v>13.52132574362516</v>
+        <v>13.52132577857056</v>
       </c>
       <c r="J132" s="2" t="n">
         <v>0.5040647235007047</v>
@@ -7460,7 +7460,7 @@
         <v>-1</v>
       </c>
       <c r="N132" s="2" t="n">
-        <v>-0.023134345253646</v>
+        <v>-0.0231343452758991</v>
       </c>
       <c r="O132" s="2" t="inlineStr">
         <is>
@@ -7481,7 +7481,7 @@
         <v/>
       </c>
       <c r="D133" s="2" t="n">
-        <v>57.71432146249276</v>
+        <v>57.7143214625001</v>
       </c>
       <c r="E133" s="2" t="n">
         <v>12.2</v>
@@ -7495,10 +7495,10 @@
         <v>0</v>
       </c>
       <c r="H133" s="2" t="n">
-        <v>45.35244733663379</v>
+        <v>45.35244724899106</v>
       </c>
       <c r="I133" s="2" t="n">
-        <v>17.19114594544309</v>
+        <v>17.19114592414732</v>
       </c>
       <c r="J133" s="2" t="n">
         <v>1.00129717614731</v>
@@ -7513,7 +7513,7 @@
         <v>-1</v>
       </c>
       <c r="N133" s="2" t="n">
-        <v>-0.0179311101640228</v>
+        <v>-0.0179311101306407</v>
       </c>
       <c r="O133" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
scan: seg0 2026-10-10 00:13 CST
</commit_message>
<xml_diff>
--- a/output/full_scan/batch_seq1_2026-10-08.xlsx
+++ b/output/full_scan/batch_seq1_2026-10-08.xlsx
@@ -552,10 +552,10 @@
         <v>0</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>80.17283677498976</v>
+        <v>80.17283670413103</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>30.21258054563315</v>
+        <v>30.21258052481157</v>
       </c>
       <c r="J2" s="2" t="n">
         <v>6.188783704430866</v>
@@ -570,7 +570,7 @@
         <v>-1</v>
       </c>
       <c r="N2" s="2" t="n">
-        <v>1.274804539808161</v>
+        <v>1.27480453996438</v>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
@@ -605,10 +605,10 @@
         <v>0</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>69.20121058570251</v>
+        <v>69.20121054348961</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>31.81656597158955</v>
+        <v>31.81656589519695</v>
       </c>
       <c r="J3" s="2" t="n">
         <v>2.784783857650602</v>
@@ -623,7 +623,7 @@
         <v>-1</v>
       </c>
       <c r="N3" s="2" t="n">
-        <v>0.752576245493159</v>
+        <v>0.752576245553235</v>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
@@ -658,10 +658,10 @@
         <v>0</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>64.73263822920607</v>
+        <v>64.73263810790868</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>38.24791131681714</v>
+        <v>38.24791130061408</v>
       </c>
       <c r="J4" s="2" t="n">
         <v>2.665352528502424</v>
@@ -676,7 +676,7 @@
         <v>-1</v>
       </c>
       <c r="N4" s="2" t="n">
-        <v>4.460652702809876</v>
+        <v>4.460652702329181</v>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
@@ -711,10 +711,10 @@
         <v>0</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>70.8906803103731</v>
+        <v>70.8906802196046</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>27.3190878604013</v>
+        <v>27.31908778846014</v>
       </c>
       <c r="J5" s="2" t="n">
         <v>4.018966822028805</v>
@@ -729,7 +729,7 @@
         <v>-1</v>
       </c>
       <c r="N5" s="2" t="n">
-        <v>0.1328052751330564</v>
+        <v>0.1328052751691074</v>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
@@ -764,10 +764,10 @@
         <v>0</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>70.51754760490209</v>
+        <v>70.51754764303104</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>41.32971167159844</v>
+        <v>41.32971171609378</v>
       </c>
       <c r="J6" s="2" t="n">
         <v>2.469735452198493</v>
@@ -782,7 +782,7 @@
         <v>-1</v>
       </c>
       <c r="N6" s="2" t="n">
-        <v>0.1112840052926858</v>
+        <v>0.111284005319126</v>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
@@ -803,7 +803,7 @@
         <v/>
       </c>
       <c r="D7" s="2" t="n">
-        <v>1075.262858764167</v>
+        <v>1075.262858764168</v>
       </c>
       <c r="E7" s="2" t="n">
         <v>12.8</v>
@@ -817,10 +817,10 @@
         <v>0</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>64.87295581596869</v>
+        <v>64.87295552989823</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>31.7885638580313</v>
+        <v>31.78856377062912</v>
       </c>
       <c r="J7" s="2" t="n">
         <v>2.169258250102063</v>
@@ -835,7 +835,7 @@
         <v>-1</v>
       </c>
       <c r="N7" s="2" t="n">
-        <v>0.0451363329956377</v>
+        <v>0.0451363331999341</v>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
@@ -856,7 +856,7 @@
         <v/>
       </c>
       <c r="D8" s="2" t="n">
-        <v>1040.908419774198</v>
+        <v>1040.908419774202</v>
       </c>
       <c r="E8" s="2" t="n">
         <v>26.95</v>
@@ -870,10 +870,10 @@
         <v>0</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>61.11680407478901</v>
+        <v>61.11680377997972</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>30.61470983579274</v>
+        <v>30.6147101737819</v>
       </c>
       <c r="J8" s="2" t="n">
         <v>3.517637716604867</v>
@@ -888,7 +888,7 @@
         <v>-1</v>
       </c>
       <c r="N8" s="2" t="n">
-        <v>0.0945599074603575</v>
+        <v>0.09455990764061489</v>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
@@ -923,10 +923,10 @@
         <v>0</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>63.69775659100706</v>
+        <v>63.69775643454888</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>23.0351335393537</v>
+        <v>23.03513358580089</v>
       </c>
       <c r="J9" s="2" t="n">
         <v>1.436548254733174</v>
@@ -941,7 +941,7 @@
         <v>-1</v>
       </c>
       <c r="N9" s="2" t="n">
-        <v>0.0135171219475053</v>
+        <v>0.0135171218874187</v>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
@@ -976,10 +976,10 @@
         <v>0</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>65.10548705143836</v>
+        <v>65.10548694265148</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>16.38585827537656</v>
+        <v>16.38585839919321</v>
       </c>
       <c r="J10" s="2" t="n">
         <v>3.207628224778093</v>
@@ -994,7 +994,7 @@
         <v>-1</v>
       </c>
       <c r="N10" s="2" t="n">
-        <v>0.0826251691176256</v>
+        <v>0.0826251692017462</v>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
@@ -1015,7 +1015,7 @@
         <v/>
       </c>
       <c r="D11" s="2" t="n">
-        <v>987.609373507877</v>
+        <v>987.6093735078772</v>
       </c>
       <c r="E11" s="2" t="n">
         <v>15.15</v>
@@ -1029,10 +1029,10 @@
         <v>0</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>60.19145462843796</v>
+        <v>60.19145461045038</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>41.95328184547853</v>
+        <v>41.95328191466345</v>
       </c>
       <c r="J11" s="2" t="n">
         <v>1.454658485441723</v>
@@ -1047,7 +1047,7 @@
         <v>-1</v>
       </c>
       <c r="N11" s="2" t="n">
-        <v>-0.0293590203607285</v>
+        <v>-0.0293590203246785</v>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
@@ -1068,7 +1068,7 @@
         <v/>
       </c>
       <c r="D12" s="2" t="n">
-        <v>986.482583861012</v>
+        <v>986.4825838610116</v>
       </c>
       <c r="E12" s="2" t="n">
         <v>13</v>
@@ -1082,10 +1082,10 @@
         <v>0</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>64.23333306825251</v>
+        <v>64.23333292933413</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>21.41760445922887</v>
+        <v>21.4176044550177</v>
       </c>
       <c r="J12" s="2" t="n">
         <v>2.010355149902084</v>
@@ -1100,7 +1100,7 @@
         <v>-1</v>
       </c>
       <c r="N12" s="2" t="n">
-        <v>0.0892334310300391</v>
+        <v>0.0892334311141583</v>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
@@ -1121,7 +1121,7 @@
         <v/>
       </c>
       <c r="D13" s="2" t="n">
-        <v>963.7132837691298</v>
+        <v>963.71328376913</v>
       </c>
       <c r="E13" s="2" t="n">
         <v>310</v>
@@ -1135,10 +1135,10 @@
         <v>0</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>76.71131973789321</v>
+        <v>76.71131968373544</v>
       </c>
       <c r="I13" s="2" t="n">
-        <v>38.78309007902674</v>
+        <v>38.78309003487535</v>
       </c>
       <c r="J13" s="2" t="n">
         <v>1.00909871808309</v>
@@ -1153,7 +1153,7 @@
         <v>-1</v>
       </c>
       <c r="N13" s="2" t="n">
-        <v>6.535923183871311</v>
+        <v>6.535923184664455</v>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
@@ -1188,10 +1188,10 @@
         <v>0</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>65.20017940538631</v>
+        <v>65.20017937265564</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>40.17082534131506</v>
+        <v>40.17082545373161</v>
       </c>
       <c r="J14" s="2" t="n">
         <v>1.086929629099419</v>
@@ -1206,7 +1206,7 @@
         <v>-1</v>
       </c>
       <c r="N14" s="2" t="n">
-        <v>0.066587503992904</v>
+        <v>0.0665875037869465</v>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
@@ -1227,7 +1227,7 @@
         <v/>
       </c>
       <c r="D15" s="2" t="n">
-        <v>904.9499122320606</v>
+        <v>904.9499122320574</v>
       </c>
       <c r="E15" s="2" t="n">
         <v>13.15</v>
@@ -1241,10 +1241,10 @@
         <v>0</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>61.96836332775541</v>
+        <v>61.9683632008517</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>30.94990296910991</v>
+        <v>30.94990300119563</v>
       </c>
       <c r="J15" s="2" t="n">
         <v>2.157008870837585</v>
@@ -1259,7 +1259,7 @@
         <v>-1</v>
       </c>
       <c r="N15" s="2" t="n">
-        <v>0.07119813266321259</v>
+        <v>0.0711981327232987</v>
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
@@ -1294,10 +1294,10 @@
         <v>0</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>66.50573525073833</v>
+        <v>66.50573516648707</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>20.56815978218407</v>
+        <v>20.56815972872801</v>
       </c>
       <c r="J16" s="2" t="n">
         <v>3.133111364994963</v>
@@ -1312,7 +1312,7 @@
         <v>-1</v>
       </c>
       <c r="N16" s="2" t="n">
-        <v>0.0573879517503264</v>
+        <v>0.0573879517743607</v>
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
@@ -1347,10 +1347,10 @@
         <v>0</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>57.35964555180122</v>
+        <v>57.35964534831564</v>
       </c>
       <c r="I17" s="2" t="n">
-        <v>15.34434762138717</v>
+        <v>15.34434768753658</v>
       </c>
       <c r="J17" s="2" t="n">
         <v>1.080194659233564</v>
@@ -1365,7 +1365,7 @@
         <v>-1</v>
       </c>
       <c r="N17" s="2" t="n">
-        <v>0.1205758214138278</v>
+        <v>0.1205758212936728</v>
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
@@ -1400,10 +1400,10 @@
         <v>0</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>61.3829870749132</v>
+        <v>61.38298700775835</v>
       </c>
       <c r="I18" s="2" t="n">
-        <v>27.63174136957435</v>
+        <v>27.63174142345719</v>
       </c>
       <c r="J18" s="2" t="n">
         <v>1.186386890906387</v>
@@ -1418,7 +1418,7 @@
         <v>-1</v>
       </c>
       <c r="N18" s="2" t="n">
-        <v>2.052998328876865</v>
+        <v>2.052998328155817</v>
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
@@ -1453,10 +1453,10 @@
         <v>0</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>80.72403162355306</v>
+        <v>80.72403165363397</v>
       </c>
       <c r="I19" s="2" t="n">
-        <v>27.24659232732654</v>
+        <v>27.24659236226395</v>
       </c>
       <c r="J19" s="2" t="n">
         <v>7.946023953740562</v>
@@ -1471,7 +1471,7 @@
         <v>-1</v>
       </c>
       <c r="N19" s="2" t="n">
-        <v>0.4156284589269245</v>
+        <v>0.4156284588908743</v>
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
@@ -1506,10 +1506,10 @@
         <v>0</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>72.06372204378749</v>
+        <v>72.06372205174338</v>
       </c>
       <c r="I20" s="2" t="n">
-        <v>49.65411203780359</v>
+        <v>49.65411204383348</v>
       </c>
       <c r="J20" s="2" t="n">
         <v>0.2516352881706286</v>
@@ -1524,7 +1524,7 @@
         <v>-1</v>
       </c>
       <c r="N20" s="2" t="n">
-        <v>7.149312460588476</v>
+        <v>7.149312461069044</v>
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
@@ -1559,10 +1559,10 @@
         <v>0</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>74.21164350091702</v>
+        <v>74.21164357167467</v>
       </c>
       <c r="I21" s="2" t="n">
-        <v>62.99566189791751</v>
+        <v>62.99566196241483</v>
       </c>
       <c r="J21" s="2" t="n">
         <v>0.9414565960544968</v>
@@ -1577,7 +1577,7 @@
         <v>-1</v>
       </c>
       <c r="N21" s="2" t="n">
-        <v>0.8359666324711732</v>
+        <v>0.8359666323510062</v>
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
@@ -1598,7 +1598,7 @@
         <v/>
       </c>
       <c r="D22" s="2" t="n">
-        <v>775.5124576916787</v>
+        <v>775.5124576916786</v>
       </c>
       <c r="E22" s="2" t="n">
         <v>14.55</v>
@@ -1612,10 +1612,10 @@
         <v>0</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>55.31063553190197</v>
+        <v>55.31063539707024</v>
       </c>
       <c r="I22" s="2" t="n">
-        <v>34.7994550079277</v>
+        <v>34.79945503038725</v>
       </c>
       <c r="J22" s="2" t="n">
         <v>1.203460007458598</v>
@@ -1630,7 +1630,7 @@
         <v>-1</v>
       </c>
       <c r="N22" s="2" t="n">
-        <v>0.022626734701186</v>
+        <v>0.0226267347732906</v>
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
@@ -1651,7 +1651,7 @@
         <v/>
       </c>
       <c r="D23" s="2" t="n">
-        <v>772.0867034366441</v>
+        <v>772.086703436644</v>
       </c>
       <c r="E23" s="2" t="n">
         <v>72.8</v>
@@ -1665,10 +1665,10 @@
         <v>0</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>86.12733784641473</v>
+        <v>86.12733786684265</v>
       </c>
       <c r="I23" s="2" t="n">
-        <v>47.95825927001134</v>
+        <v>47.95825930827112</v>
       </c>
       <c r="J23" s="2" t="n">
         <v>2.478770809180932</v>
@@ -1683,7 +1683,7 @@
         <v>-1</v>
       </c>
       <c r="N23" s="2" t="n">
-        <v>0.3896946648677832</v>
+        <v>0.3896946648197148</v>
       </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
@@ -1721,7 +1721,7 @@
         <v>58.35918143127039</v>
       </c>
       <c r="I24" s="2" t="n">
-        <v>22.35063832506045</v>
+        <v>22.35063828600368</v>
       </c>
       <c r="J24" s="2" t="n">
         <v>0.8137865049238459</v>
@@ -1771,10 +1771,10 @@
         <v>0</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>60.78707803637715</v>
+        <v>60.78707798091916</v>
       </c>
       <c r="I25" s="2" t="n">
-        <v>41.19635168365246</v>
+        <v>41.19635162093068</v>
       </c>
       <c r="J25" s="2" t="n">
         <v>1.101693581738865</v>
@@ -1789,7 +1789,7 @@
         <v>-1</v>
       </c>
       <c r="N25" s="2" t="n">
-        <v>-0.0009089541716004</v>
+        <v>-0.0009089541379506</v>
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
@@ -1824,10 +1824,10 @@
         <v>0</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>53.5603180470249</v>
+        <v>53.560317624215</v>
       </c>
       <c r="I26" s="2" t="n">
-        <v>23.68266746806872</v>
+        <v>23.68266749033058</v>
       </c>
       <c r="J26" s="2" t="n">
         <v>0.4614597553978389</v>
@@ -1863,7 +1863,7 @@
         <v/>
       </c>
       <c r="D27" s="2" t="n">
-        <v>706.9453848837487</v>
+        <v>706.9453848837501</v>
       </c>
       <c r="E27" s="2" t="n">
         <v>25.8</v>
@@ -1877,10 +1877,10 @@
         <v>0</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>53.88024028272982</v>
+        <v>53.88024029762013</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>31.535091878016</v>
+        <v>31.53509193744399</v>
       </c>
       <c r="J27" s="2" t="n">
         <v>0.5260641077467636</v>
@@ -1895,7 +1895,7 @@
         <v>-1</v>
       </c>
       <c r="N27" s="2" t="n">
-        <v>0.0431057183160886</v>
+        <v>0.0431057182800353</v>
       </c>
       <c r="O27" s="2" t="inlineStr">
         <is>
@@ -1916,7 +1916,7 @@
         <v/>
       </c>
       <c r="D28" s="2" t="n">
-        <v>697.2854171379375</v>
+        <v>697.2854171379372</v>
       </c>
       <c r="E28" s="2" t="n">
         <v>167</v>
@@ -1930,10 +1930,10 @@
         <v>0</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>52.74449371447933</v>
+        <v>52.74449360460171</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>8.543380743916792</v>
+        <v>8.543380787219393</v>
       </c>
       <c r="J28" s="2" t="n">
         <v>0.8309668319414185</v>
@@ -1948,7 +1948,7 @@
         <v>-1</v>
       </c>
       <c r="N28" s="2" t="n">
-        <v>0.1117792673928514</v>
+        <v>0.1117792678735815</v>
       </c>
       <c r="O28" s="2" t="inlineStr">
         <is>
@@ -1969,7 +1969,7 @@
         <v/>
       </c>
       <c r="D29" s="2" t="n">
-        <v>694.5405199595455</v>
+        <v>694.5405199595451</v>
       </c>
       <c r="E29" s="2" t="n">
         <v>14.35</v>
@@ -1983,10 +1983,10 @@
         <v>0</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>58.56917052687851</v>
+        <v>58.56917036948725</v>
       </c>
       <c r="I29" s="2" t="n">
-        <v>33.40026644958505</v>
+        <v>33.40026654357774</v>
       </c>
       <c r="J29" s="2" t="n">
         <v>1.092231304575591</v>
@@ -2001,7 +2001,7 @@
         <v>-1</v>
       </c>
       <c r="N29" s="2" t="n">
-        <v>0.0467512310527251</v>
+        <v>0.0467512311488649</v>
       </c>
       <c r="O29" s="2" t="inlineStr">
         <is>
@@ -2036,10 +2036,10 @@
         <v>0</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>54.45660325701563</v>
+        <v>54.45660331046034</v>
       </c>
       <c r="I30" s="2" t="n">
-        <v>13.78446990000659</v>
+        <v>13.7844699316857</v>
       </c>
       <c r="J30" s="2" t="n">
         <v>1.077817835173378</v>
@@ -2054,7 +2054,7 @@
         <v>-1</v>
       </c>
       <c r="N30" s="2" t="n">
-        <v>0.1306838959506828</v>
+        <v>0.1306838957103338</v>
       </c>
       <c r="O30" s="2" t="inlineStr">
         <is>
@@ -2089,10 +2089,10 @@
         <v>0</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>58.40651283713011</v>
+        <v>58.40651268624093</v>
       </c>
       <c r="I31" s="2" t="n">
-        <v>39.62181534004888</v>
+        <v>39.62181531058651</v>
       </c>
       <c r="J31" s="2" t="n">
         <v>0.8969147358565098</v>
@@ -2107,7 +2107,7 @@
         <v>-1</v>
       </c>
       <c r="N31" s="2" t="n">
-        <v>0.0543106075261421</v>
+        <v>0.0543106075742114</v>
       </c>
       <c r="O31" s="2" t="inlineStr">
         <is>
@@ -2128,7 +2128,7 @@
         <v/>
       </c>
       <c r="D32" s="2" t="n">
-        <v>686.9023908853081</v>
+        <v>686.9023908853072</v>
       </c>
       <c r="E32" s="2" t="n">
         <v>71.7</v>
@@ -2142,10 +2142,10 @@
         <v>0</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>56.25975825916096</v>
+        <v>56.25975803986667</v>
       </c>
       <c r="I32" s="2" t="n">
-        <v>15.98731785562862</v>
+        <v>15.98731791096328</v>
       </c>
       <c r="J32" s="2" t="n">
         <v>1.715354894706094</v>
@@ -2160,7 +2160,7 @@
         <v>-1</v>
       </c>
       <c r="N32" s="2" t="n">
-        <v>0.3252857665325743</v>
+        <v>0.3252857672536181</v>
       </c>
       <c r="O32" s="2" t="inlineStr">
         <is>
@@ -2198,7 +2198,7 @@
         <v>56.6201698096582</v>
       </c>
       <c r="I33" s="2" t="n">
-        <v>31.85762139324562</v>
+        <v>31.85762141188791</v>
       </c>
       <c r="J33" s="2" t="n">
         <v>4.219483892167547</v>
@@ -2213,7 +2213,7 @@
         <v>-1</v>
       </c>
       <c r="N33" s="2" t="n">
-        <v>0.0623421480774131</v>
+        <v>0.0623421480822184</v>
       </c>
       <c r="O33" s="2" t="inlineStr">
         <is>
@@ -2248,10 +2248,10 @@
         <v>0</v>
       </c>
       <c r="H34" s="2" t="n">
-        <v>55.72431513553103</v>
+        <v>55.72431509181454</v>
       </c>
       <c r="I34" s="2" t="n">
-        <v>8.516846101263933</v>
+        <v>8.516846054118014</v>
       </c>
       <c r="J34" s="2" t="n">
         <v>1.134325838571727</v>
@@ -2287,7 +2287,7 @@
         <v/>
       </c>
       <c r="D35" s="2" t="n">
-        <v>664.8039400019213</v>
+        <v>664.803940001921</v>
       </c>
       <c r="E35" s="2" t="n">
         <v>26.05</v>
@@ -2301,10 +2301,10 @@
         <v>0</v>
       </c>
       <c r="H35" s="2" t="n">
-        <v>61.1456356822364</v>
+        <v>61.14563551406447</v>
       </c>
       <c r="I35" s="2" t="n">
-        <v>19.87545071030605</v>
+        <v>19.87545062150313</v>
       </c>
       <c r="J35" s="2" t="n">
         <v>0.9964773310473706</v>
@@ -2319,7 +2319,7 @@
         <v>-1</v>
       </c>
       <c r="N35" s="2" t="n">
-        <v>0.1748588758780659</v>
+        <v>0.1748588762626225</v>
       </c>
       <c r="O35" s="2" t="inlineStr">
         <is>
@@ -2354,10 +2354,10 @@
         <v>0</v>
       </c>
       <c r="H36" s="2" t="n">
-        <v>56.08314226584429</v>
+        <v>56.08314228753697</v>
       </c>
       <c r="I36" s="2" t="n">
-        <v>15.88962155302476</v>
+        <v>15.889621745958</v>
       </c>
       <c r="J36" s="2" t="n">
         <v>0.3399736555728307</v>
@@ -2393,7 +2393,7 @@
         <v/>
       </c>
       <c r="D37" s="2" t="n">
-        <v>573.5987391508008</v>
+        <v>573.598739150801</v>
       </c>
       <c r="E37" s="2" t="n">
         <v>18.65</v>
@@ -2407,10 +2407,10 @@
         <v>0</v>
       </c>
       <c r="H37" s="2" t="n">
-        <v>62.36392639714726</v>
+        <v>62.36392620791799</v>
       </c>
       <c r="I37" s="2" t="n">
-        <v>35.65574021052848</v>
+        <v>35.65574017592879</v>
       </c>
       <c r="J37" s="2" t="n">
         <v>0.5176600408040768</v>
@@ -2425,7 +2425,7 @@
         <v>-1</v>
       </c>
       <c r="N37" s="2" t="n">
-        <v>0.0943121665042737</v>
+        <v>0.0943121664802353</v>
       </c>
       <c r="O37" s="2" t="inlineStr">
         <is>
@@ -2460,10 +2460,10 @@
         <v>0</v>
       </c>
       <c r="H38" s="2" t="n">
-        <v>56.31338572741889</v>
+        <v>56.31338569339808</v>
       </c>
       <c r="I38" s="2" t="n">
-        <v>37.18109046029698</v>
+        <v>37.18109075439504</v>
       </c>
       <c r="J38" s="2" t="n">
         <v>0.2343401662160509</v>
@@ -2478,7 +2478,7 @@
         <v>-1</v>
       </c>
       <c r="N38" s="2" t="n">
-        <v>0.0618683372622511</v>
+        <v>0.0618683372862865</v>
       </c>
       <c r="O38" s="2" t="inlineStr">
         <is>
@@ -2513,10 +2513,10 @@
         <v>0</v>
       </c>
       <c r="H39" s="2" t="n">
-        <v>47.37128773022167</v>
+        <v>47.37128756230537</v>
       </c>
       <c r="I39" s="2" t="n">
-        <v>37.23378493046936</v>
+        <v>37.23378492537553</v>
       </c>
       <c r="J39" s="2" t="n">
         <v>0.4176033749544254</v>
@@ -2531,7 +2531,7 @@
         <v>-1</v>
       </c>
       <c r="N39" s="2" t="n">
-        <v>-0.8541210191535056</v>
+        <v>-0.8541210187929975</v>
       </c>
       <c r="O39" s="2" t="inlineStr">
         <is>
@@ -2566,10 +2566,10 @@
         <v>0</v>
       </c>
       <c r="H40" s="2" t="n">
-        <v>58.87775263406078</v>
+        <v>58.8777528238077</v>
       </c>
       <c r="I40" s="2" t="n">
-        <v>19.4801625473852</v>
+        <v>19.48016264736069</v>
       </c>
       <c r="J40" s="2" t="n">
         <v>1.44946356748814</v>
@@ -2584,7 +2584,7 @@
         <v>-1</v>
       </c>
       <c r="N40" s="2" t="n">
-        <v>0.0545869841164134</v>
+        <v>0.0545869840563262</v>
       </c>
       <c r="O40" s="2" t="inlineStr">
         <is>
@@ -2619,10 +2619,10 @@
         <v>0</v>
       </c>
       <c r="H41" s="2" t="n">
-        <v>53.1575712220322</v>
+        <v>53.1575711909082</v>
       </c>
       <c r="I41" s="2" t="n">
-        <v>11.6876762182732</v>
+        <v>11.68767615003111</v>
       </c>
       <c r="J41" s="2" t="n">
         <v>0.556293488945834</v>
@@ -2637,7 +2637,7 @@
         <v>-1</v>
       </c>
       <c r="N41" s="2" t="n">
-        <v>0.0362735806158178</v>
+        <v>0.0362735806278317</v>
       </c>
       <c r="O41" s="2" t="inlineStr">
         <is>
@@ -2672,10 +2672,10 @@
         <v>0</v>
       </c>
       <c r="H42" s="2" t="n">
-        <v>52.65346415520652</v>
+        <v>52.65346391545582</v>
       </c>
       <c r="I42" s="2" t="n">
-        <v>37.46372394343865</v>
+        <v>37.46372419638679</v>
       </c>
       <c r="J42" s="2" t="n">
         <v>0.2010716673320789</v>
@@ -2690,7 +2690,7 @@
         <v>-1</v>
       </c>
       <c r="N42" s="2" t="n">
-        <v>-0.3110437947313542</v>
+        <v>-0.3110437942626765</v>
       </c>
       <c r="O42" s="2" t="inlineStr">
         <is>
@@ -2725,10 +2725,10 @@
         <v>0</v>
       </c>
       <c r="H43" s="2" t="n">
-        <v>56.55829453134284</v>
+        <v>56.55829447599088</v>
       </c>
       <c r="I43" s="2" t="n">
-        <v>20.97914438166865</v>
+        <v>20.97914422234292</v>
       </c>
       <c r="J43" s="2" t="n">
         <v>1.650945095700728</v>
@@ -2743,7 +2743,7 @@
         <v>-1</v>
       </c>
       <c r="N43" s="2" t="n">
-        <v>0.0284657122319598</v>
+        <v>0.0284657122439768</v>
       </c>
       <c r="O43" s="2" t="inlineStr">
         <is>
@@ -2778,10 +2778,10 @@
         <v>0</v>
       </c>
       <c r="H44" s="2" t="n">
-        <v>51.14189599676926</v>
+        <v>51.14189599393909</v>
       </c>
       <c r="I44" s="2" t="n">
-        <v>21.96475352209658</v>
+        <v>21.96475356182492</v>
       </c>
       <c r="J44" s="2" t="n">
         <v>1.783222894230914</v>
@@ -2796,7 +2796,7 @@
         <v>-1</v>
       </c>
       <c r="N44" s="2" t="n">
-        <v>-1.0901459017569</v>
+        <v>-1.090145901708834</v>
       </c>
       <c r="O44" s="2" t="inlineStr">
         <is>
@@ -2834,7 +2834,7 @@
         <v>39.1196293527881</v>
       </c>
       <c r="I45" s="2" t="n">
-        <v>27.07119763782859</v>
+        <v>27.0711975940465</v>
       </c>
       <c r="J45" s="2" t="n">
         <v>0.9335601920955612</v>
@@ -2849,7 +2849,7 @@
         <v>-1</v>
       </c>
       <c r="N45" s="2" t="n">
-        <v>-0.0049953932691792</v>
+        <v>-0.0049953933653184</v>
       </c>
       <c r="O45" s="2" t="inlineStr">
         <is>
@@ -2884,10 +2884,10 @@
         <v>0</v>
       </c>
       <c r="H46" s="2" t="n">
-        <v>52.40347475732364</v>
+        <v>52.40347474358145</v>
       </c>
       <c r="I46" s="2" t="n">
-        <v>4.726421381427445</v>
+        <v>4.726421488483217</v>
       </c>
       <c r="J46" s="2" t="n">
         <v>1.443319884863796</v>
@@ -2902,7 +2902,7 @@
         <v>-1</v>
       </c>
       <c r="N46" s="2" t="n">
-        <v>0.0310364302309483</v>
+        <v>0.0310364302189311</v>
       </c>
       <c r="O46" s="2" t="inlineStr">
         <is>
@@ -2937,10 +2937,10 @@
         <v>0</v>
       </c>
       <c r="H47" s="2" t="n">
-        <v>64.70140804958056</v>
+        <v>64.70140799437485</v>
       </c>
       <c r="I47" s="2" t="n">
-        <v>62.17497344573913</v>
+        <v>62.17497330663279</v>
       </c>
       <c r="J47" s="2" t="n">
         <v>0.6355803468523609</v>
@@ -2955,7 +2955,7 @@
         <v>-1</v>
       </c>
       <c r="N47" s="2" t="n">
-        <v>0.2138992901195479</v>
+        <v>0.2138992901607393</v>
       </c>
       <c r="O47" s="2" t="inlineStr">
         <is>
@@ -2990,10 +2990,10 @@
         <v>0</v>
       </c>
       <c r="H48" s="2" t="n">
-        <v>51.10274972091622</v>
+        <v>51.10274970811394</v>
       </c>
       <c r="I48" s="2" t="n">
-        <v>12.10792045513235</v>
+        <v>12.10792047991298</v>
       </c>
       <c r="J48" s="2" t="n">
         <v>0.6754374092350689</v>
@@ -3008,7 +3008,7 @@
         <v>-1</v>
       </c>
       <c r="N48" s="2" t="n">
-        <v>0.0870757644684919</v>
+        <v>0.08707576448050861</v>
       </c>
       <c r="O48" s="2" t="inlineStr">
         <is>
@@ -3043,10 +3043,10 @@
         <v>0</v>
       </c>
       <c r="H49" s="2" t="n">
-        <v>59.29428232067028</v>
+        <v>59.29428233902889</v>
       </c>
       <c r="I49" s="2" t="n">
-        <v>13.52922294901413</v>
+        <v>13.52922298869362</v>
       </c>
       <c r="J49" s="2" t="n">
         <v>0.244590014339721</v>
@@ -3061,7 +3061,7 @@
         <v>-1</v>
       </c>
       <c r="N49" s="2" t="n">
-        <v>0.7751930105089038</v>
+        <v>0.775193010400748</v>
       </c>
       <c r="O49" s="2" t="inlineStr">
         <is>
@@ -3096,10 +3096,10 @@
         <v>0</v>
       </c>
       <c r="H50" s="2" t="n">
-        <v>48.75497590505417</v>
+        <v>48.75497588524127</v>
       </c>
       <c r="I50" s="2" t="n">
-        <v>17.65773684976121</v>
+        <v>17.65773693562737</v>
       </c>
       <c r="J50" s="2" t="n">
         <v>0.9171836345490876</v>
@@ -3114,7 +3114,7 @@
         <v>-1</v>
       </c>
       <c r="N50" s="2" t="n">
-        <v>0.1737957924339361</v>
+        <v>0.1737957924579791</v>
       </c>
       <c r="O50" s="2" t="inlineStr">
         <is>
@@ -3149,10 +3149,10 @@
         <v>0</v>
       </c>
       <c r="H51" s="2" t="n">
-        <v>49.55989816423709</v>
+        <v>49.55989814796669</v>
       </c>
       <c r="I51" s="2" t="n">
-        <v>14.82984346640293</v>
+        <v>14.82984333650718</v>
       </c>
       <c r="J51" s="2" t="n">
         <v>0.5977558243061</v>
@@ -3167,7 +3167,7 @@
         <v>-1</v>
       </c>
       <c r="N51" s="2" t="n">
-        <v>0.0414281014252889</v>
+        <v>0.0414281014300972</v>
       </c>
       <c r="O51" s="2" t="inlineStr">
         <is>
@@ -3202,10 +3202,10 @@
         <v>0</v>
       </c>
       <c r="H52" s="2" t="n">
-        <v>52.48147513693962</v>
+        <v>52.4814740791379</v>
       </c>
       <c r="I52" s="2" t="n">
-        <v>8.649900945101788</v>
+        <v>8.649900893500625</v>
       </c>
       <c r="J52" s="2" t="n">
         <v>0.4090731176431278</v>
@@ -3255,10 +3255,10 @@
         <v>0</v>
       </c>
       <c r="H53" s="2" t="n">
-        <v>53.77245546858805</v>
+        <v>53.77245455229886</v>
       </c>
       <c r="I53" s="2" t="n">
-        <v>19.59757051352537</v>
+        <v>19.59757079932205</v>
       </c>
       <c r="J53" s="2" t="n">
         <v>0.7354925662724614</v>
@@ -3273,7 +3273,7 @@
         <v>-1</v>
       </c>
       <c r="N53" s="2" t="n">
-        <v>0.0090334233611363</v>
+        <v>0.009033423397187899</v>
       </c>
       <c r="O53" s="2" t="inlineStr">
         <is>
@@ -3294,7 +3294,7 @@
         <v/>
       </c>
       <c r="D54" s="2" t="n">
-        <v>395.7555989745435</v>
+        <v>395.7555989745423</v>
       </c>
       <c r="E54" s="2" t="n">
         <v>17.15</v>
@@ -3308,7 +3308,7 @@
         <v>0</v>
       </c>
       <c r="H54" s="2" t="n">
-        <v>52.50674126073569</v>
+        <v>52.50674131666343</v>
       </c>
       <c r="I54" s="2" t="n">
         <v>18.11407924387222</v>
@@ -3326,7 +3326,7 @@
         <v>-1</v>
       </c>
       <c r="N54" s="2" t="n">
-        <v>0.0134957593245204</v>
+        <v>0.0134957592884673</v>
       </c>
       <c r="O54" s="2" t="inlineStr">
         <is>
@@ -3361,10 +3361,10 @@
         <v>0</v>
       </c>
       <c r="H55" s="2" t="n">
-        <v>53.51103909936661</v>
+        <v>53.51103910329788</v>
       </c>
       <c r="I55" s="2" t="n">
-        <v>8.456234704761002</v>
+        <v>8.456234704761</v>
       </c>
       <c r="J55" s="2" t="n">
         <v>0.5690058807924451</v>
@@ -3379,7 +3379,7 @@
         <v>-1</v>
       </c>
       <c r="N55" s="2" t="n">
-        <v>0.9405787507265928</v>
+        <v>0.9405787505823812</v>
       </c>
       <c r="O55" s="2" t="inlineStr">
         <is>
@@ -3400,7 +3400,7 @@
         <v/>
       </c>
       <c r="D56" s="2" t="n">
-        <v>389.5086574968054</v>
+        <v>389.5086574968053</v>
       </c>
       <c r="E56" s="2" t="n">
         <v>13.15</v>
@@ -3417,7 +3417,7 @@
         <v>50.20325719991721</v>
       </c>
       <c r="I56" s="2" t="n">
-        <v>25.41589931029747</v>
+        <v>25.41589916349009</v>
       </c>
       <c r="J56" s="2" t="n">
         <v>0.8476163592073097</v>
@@ -3432,7 +3432,7 @@
         <v>-1</v>
       </c>
       <c r="N56" s="2" t="n">
-        <v>0.0067909159990324</v>
+        <v>0.0067909159749979</v>
       </c>
       <c r="O56" s="2" t="inlineStr">
         <is>
@@ -3467,10 +3467,10 @@
         <v>0</v>
       </c>
       <c r="H57" s="2" t="n">
-        <v>54.63154497065917</v>
+        <v>54.63154487395931</v>
       </c>
       <c r="I57" s="2" t="n">
-        <v>16.82689286159843</v>
+        <v>16.82689290638939</v>
       </c>
       <c r="J57" s="2" t="n">
         <v>1.021403050383265</v>
@@ -3485,7 +3485,7 @@
         <v>-1</v>
       </c>
       <c r="N57" s="2" t="n">
-        <v>0.0195329586852375</v>
+        <v>0.0195329586972562</v>
       </c>
       <c r="O57" s="2" t="inlineStr">
         <is>
@@ -3506,7 +3506,7 @@
         <v/>
       </c>
       <c r="D58" s="2" t="n">
-        <v>386.0804565903412</v>
+        <v>386.0804565903411</v>
       </c>
       <c r="E58" s="2" t="n">
         <v>24.2</v>
@@ -3520,10 +3520,10 @@
         <v>0</v>
       </c>
       <c r="H58" s="2" t="n">
-        <v>51.86276959606941</v>
+        <v>51.8627721404521</v>
       </c>
       <c r="I58" s="2" t="n">
-        <v>8.884628207476135</v>
+        <v>8.884629373789879</v>
       </c>
       <c r="J58" s="2" t="n">
         <v>0.2012828426504924</v>
@@ -3538,7 +3538,7 @@
         <v>-1</v>
       </c>
       <c r="N58" s="2" t="n">
-        <v>-0.009139085983431</v>
+        <v>-0.0091390908504379</v>
       </c>
       <c r="O58" s="2" t="inlineStr">
         <is>
@@ -3573,10 +3573,10 @@
         <v>0</v>
       </c>
       <c r="H59" s="2" t="n">
-        <v>55.38532481591836</v>
+        <v>55.38532480139908</v>
       </c>
       <c r="I59" s="2" t="n">
-        <v>12.63650291873043</v>
+        <v>12.63650282874752</v>
       </c>
       <c r="J59" s="2" t="n">
         <v>0.6892411045184866</v>
@@ -3591,7 +3591,7 @@
         <v>-1</v>
       </c>
       <c r="N59" s="2" t="n">
-        <v>0.0942736518691895</v>
+        <v>0.09427365179708409</v>
       </c>
       <c r="O59" s="2" t="inlineStr">
         <is>
@@ -3644,7 +3644,7 @@
         <v>-1</v>
       </c>
       <c r="N60" s="2" t="n">
-        <v>0.0715501358574048</v>
+        <v>0.0715501358383346</v>
       </c>
       <c r="O60" s="2" t="inlineStr">
         <is>
@@ -3679,10 +3679,10 @@
         <v>0</v>
       </c>
       <c r="H61" s="2" t="n">
-        <v>35.28327272252579</v>
+        <v>35.28327243731648</v>
       </c>
       <c r="I61" s="2" t="n">
-        <v>46.92575169544239</v>
+        <v>46.92575180509017</v>
       </c>
       <c r="J61" s="2" t="n">
         <v>0.3770570139760966</v>
@@ -3697,7 +3697,7 @@
         <v>-1</v>
       </c>
       <c r="N61" s="2" t="n">
-        <v>0.0347248429943436</v>
+        <v>0.0347248430303946</v>
       </c>
       <c r="O61" s="2" t="inlineStr">
         <is>
@@ -3735,7 +3735,7 @@
         <v>48.04021488424984</v>
       </c>
       <c r="I62" s="2" t="n">
-        <v>18.79509926542985</v>
+        <v>18.79509927018536</v>
       </c>
       <c r="J62" s="2" t="n">
         <v>1.622855482725268</v>
@@ -3750,7 +3750,7 @@
         <v>-1</v>
       </c>
       <c r="N62" s="2" t="n">
-        <v>0.0324822900559068</v>
+        <v>0.0324822900679242</v>
       </c>
       <c r="O62" s="2" t="inlineStr">
         <is>
@@ -3788,7 +3788,7 @@
         <v>46.50061881716901</v>
       </c>
       <c r="I63" s="2" t="n">
-        <v>8.016446644399693</v>
+        <v>8.016446689695439</v>
       </c>
       <c r="J63" s="2" t="n">
         <v>0.7693891200315155</v>
@@ -3803,7 +3803,7 @@
         <v>-1</v>
       </c>
       <c r="N63" s="2" t="n">
-        <v>0.2246841619158339</v>
+        <v>0.2246841622763429</v>
       </c>
       <c r="O63" s="2" t="inlineStr">
         <is>
@@ -3838,10 +3838,10 @@
         <v>0</v>
       </c>
       <c r="H64" s="2" t="n">
-        <v>37.88640013293856</v>
+        <v>37.88639928092751</v>
       </c>
       <c r="I64" s="2" t="n">
-        <v>33.46620779888283</v>
+        <v>33.46620795398771</v>
       </c>
       <c r="J64" s="2" t="n">
         <v>0.9406473455607608</v>
@@ -3856,7 +3856,7 @@
         <v>-1</v>
       </c>
       <c r="N64" s="2" t="n">
-        <v>0.1364726272729277</v>
+        <v>0.1364726275132721</v>
       </c>
       <c r="O64" s="2" t="inlineStr">
         <is>
@@ -3891,10 +3891,10 @@
         <v>0</v>
       </c>
       <c r="H65" s="2" t="n">
-        <v>45.13722423387938</v>
+        <v>45.13722421402262</v>
       </c>
       <c r="I65" s="2" t="n">
-        <v>17.4099317759493</v>
+        <v>17.4099319232083</v>
       </c>
       <c r="J65" s="2" t="n">
         <v>1.411806936854226</v>
@@ -3909,7 +3909,7 @@
         <v>-1</v>
       </c>
       <c r="N65" s="2" t="n">
-        <v>-0.034155573131642</v>
+        <v>-0.0341555731676928</v>
       </c>
       <c r="O65" s="2" t="inlineStr">
         <is>
@@ -3944,10 +3944,10 @@
         <v>0</v>
       </c>
       <c r="H66" s="2" t="n">
-        <v>47.72288222040269</v>
+        <v>47.72288171866142</v>
       </c>
       <c r="I66" s="2" t="n">
-        <v>28.92035837314694</v>
+        <v>28.92035848087663</v>
       </c>
       <c r="J66" s="2" t="n">
         <v>1.403074169411461</v>
@@ -3962,7 +3962,7 @@
         <v>-1</v>
       </c>
       <c r="N66" s="2" t="n">
-        <v>0.0190583220976972</v>
+        <v>0.0190583221938363</v>
       </c>
       <c r="O66" s="2" t="inlineStr">
         <is>
@@ -3997,10 +3997,10 @@
         <v>0</v>
       </c>
       <c r="H67" s="2" t="n">
-        <v>44.90296660626093</v>
+        <v>44.90296653229378</v>
       </c>
       <c r="I67" s="2" t="n">
-        <v>11.03991005741066</v>
+        <v>11.03991006410688</v>
       </c>
       <c r="J67" s="2" t="n">
         <v>0.6663400244064923</v>
@@ -4015,7 +4015,7 @@
         <v>-1</v>
       </c>
       <c r="N67" s="2" t="n">
-        <v>-0.0058516856593089</v>
+        <v>-0.005851685652098</v>
       </c>
       <c r="O67" s="2" t="inlineStr">
         <is>
@@ -4050,10 +4050,10 @@
         <v>0</v>
       </c>
       <c r="H68" s="2" t="n">
-        <v>42.78579994017417</v>
+        <v>42.78579987452757</v>
       </c>
       <c r="I68" s="2" t="n">
-        <v>7.411525866662092</v>
+        <v>7.411525921887339</v>
       </c>
       <c r="J68" s="2" t="n">
         <v>1.64993533516396</v>
@@ -4068,7 +4068,7 @@
         <v>-1</v>
       </c>
       <c r="N68" s="2" t="n">
-        <v>-0.0004846928860557</v>
+        <v>-0.0004846928379885</v>
       </c>
       <c r="O68" s="2" t="inlineStr">
         <is>
@@ -4103,10 +4103,10 @@
         <v>0</v>
       </c>
       <c r="H69" s="2" t="n">
-        <v>41.71233596904722</v>
+        <v>41.71233602938425</v>
       </c>
       <c r="I69" s="2" t="n">
-        <v>15.84257611083498</v>
+        <v>15.842576272444</v>
       </c>
       <c r="J69" s="2" t="n">
         <v>1.723688155693854</v>
@@ -4121,7 +4121,7 @@
         <v>-1</v>
       </c>
       <c r="N69" s="2" t="n">
-        <v>0.0062445727262468</v>
+        <v>0.0062445727022123</v>
       </c>
       <c r="O69" s="2" t="inlineStr">
         <is>
@@ -4156,10 +4156,10 @@
         <v>0</v>
       </c>
       <c r="H70" s="2" t="n">
-        <v>44.14488045828641</v>
+        <v>44.14488030173571</v>
       </c>
       <c r="I70" s="2" t="n">
-        <v>20.86074912367117</v>
+        <v>20.8607493560434</v>
       </c>
       <c r="J70" s="2" t="n">
         <v>0.7910018241300343</v>
@@ -4174,7 +4174,7 @@
         <v>-1</v>
       </c>
       <c r="N70" s="2" t="n">
-        <v>-0.0173560272057868</v>
+        <v>-0.0173560270135129</v>
       </c>
       <c r="O70" s="2" t="inlineStr">
         <is>
@@ -4209,10 +4209,10 @@
         <v>0</v>
       </c>
       <c r="H71" s="2" t="n">
-        <v>48.07630339490873</v>
+        <v>48.07630327640187</v>
       </c>
       <c r="I71" s="2" t="n">
-        <v>7.753289027694827</v>
+        <v>7.753288991094715</v>
       </c>
       <c r="J71" s="2" t="n">
         <v>0.6464284826334502</v>
@@ -4248,7 +4248,7 @@
         <v/>
       </c>
       <c r="D72" s="2" t="n">
-        <v>303.690647745484</v>
+        <v>303.6906477454838</v>
       </c>
       <c r="E72" s="2" t="n">
         <v>9.93</v>
@@ -4262,10 +4262,10 @@
         <v>0</v>
       </c>
       <c r="H72" s="2" t="n">
-        <v>39.84511966442652</v>
+        <v>39.84511974000464</v>
       </c>
       <c r="I72" s="2" t="n">
-        <v>23.42096220064119</v>
+        <v>23.42096201997182</v>
       </c>
       <c r="J72" s="2" t="n">
         <v>0.5894821430289965</v>
@@ -4280,7 +4280,7 @@
         <v>-1</v>
       </c>
       <c r="N72" s="2" t="n">
-        <v>0.0072889284278829</v>
+        <v>0.0072889284038476</v>
       </c>
       <c r="O72" s="2" t="inlineStr">
         <is>
@@ -4315,10 +4315,10 @@
         <v>0</v>
       </c>
       <c r="H73" s="2" t="n">
-        <v>49.79633150191531</v>
+        <v>49.79633150751508</v>
       </c>
       <c r="I73" s="2" t="n">
-        <v>19.90882861141895</v>
+        <v>19.90882866754414</v>
       </c>
       <c r="J73" s="2" t="n">
         <v>0.5721402003297253</v>
@@ -4333,7 +4333,7 @@
         <v>-1</v>
       </c>
       <c r="N73" s="2" t="n">
-        <v>0.0312859273718974</v>
+        <v>0.0312859273839145</v>
       </c>
       <c r="O73" s="2" t="inlineStr">
         <is>
@@ -4368,10 +4368,10 @@
         <v>0</v>
       </c>
       <c r="H74" s="2" t="n">
-        <v>44.15346261208874</v>
+        <v>44.15346274360098</v>
       </c>
       <c r="I74" s="2" t="n">
-        <v>11.68058247187292</v>
+        <v>11.68058278525822</v>
       </c>
       <c r="J74" s="2" t="n">
         <v>0.8141012996267535</v>
@@ -4386,7 +4386,7 @@
         <v>-1</v>
       </c>
       <c r="N74" s="2" t="n">
-        <v>0.0062291216984505</v>
+        <v>0.0062291215061745</v>
       </c>
       <c r="O74" s="2" t="inlineStr">
         <is>
@@ -4407,7 +4407,7 @@
         <v/>
       </c>
       <c r="D75" s="2" t="n">
-        <v>296.7085351285135</v>
+        <v>296.7085351285127</v>
       </c>
       <c r="E75" s="2" t="n">
         <v>102.5</v>
@@ -4421,10 +4421,10 @@
         <v>0</v>
       </c>
       <c r="H75" s="2" t="n">
-        <v>50.19395687493842</v>
+        <v>50.19395667197882</v>
       </c>
       <c r="I75" s="2" t="n">
-        <v>12.77439717355541</v>
+        <v>12.77439716920247</v>
       </c>
       <c r="J75" s="2" t="n">
         <v>0.8117532903989719</v>
@@ -4439,7 +4439,7 @@
         <v>-1</v>
       </c>
       <c r="N75" s="2" t="n">
-        <v>0.2006751466696338</v>
+        <v>0.2006751470301457</v>
       </c>
       <c r="O75" s="2" t="inlineStr">
         <is>
@@ -4474,10 +4474,10 @@
         <v>0</v>
       </c>
       <c r="H76" s="2" t="n">
-        <v>38.18794992498007</v>
+        <v>38.18794988483754</v>
       </c>
       <c r="I76" s="2" t="n">
-        <v>13.70238417726834</v>
+        <v>13.70238421497289</v>
       </c>
       <c r="J76" s="2" t="n">
         <v>0.2663787681529267</v>
@@ -4492,7 +4492,7 @@
         <v>-1</v>
       </c>
       <c r="N76" s="2" t="n">
-        <v>-0.1785192374331628</v>
+        <v>-0.1785192374091277</v>
       </c>
       <c r="O76" s="2" t="inlineStr">
         <is>
@@ -4513,7 +4513,7 @@
         <v/>
       </c>
       <c r="D77" s="2" t="n">
-        <v>294.1304970482884</v>
+        <v>294.1304970482883</v>
       </c>
       <c r="E77" s="2" t="n">
         <v>71.09999999999999</v>
@@ -4527,10 +4527,10 @@
         <v>0</v>
       </c>
       <c r="H77" s="2" t="n">
-        <v>46.31372200022329</v>
+        <v>46.3137218691759</v>
       </c>
       <c r="I77" s="2" t="n">
-        <v>18.96537150629971</v>
+        <v>18.9653715820402</v>
       </c>
       <c r="J77" s="2" t="n">
         <v>0.8132228938138945</v>
@@ -4545,7 +4545,7 @@
         <v>-1</v>
       </c>
       <c r="N77" s="2" t="n">
-        <v>0.2238926916976975</v>
+        <v>0.2238926918899613</v>
       </c>
       <c r="O77" s="2" t="inlineStr">
         <is>
@@ -4566,7 +4566,7 @@
         <v/>
       </c>
       <c r="D78" s="2" t="n">
-        <v>290.5806475911313</v>
+        <v>290.5806475911314</v>
       </c>
       <c r="E78" s="2" t="n">
         <v>59.1</v>
@@ -4580,10 +4580,10 @@
         <v>0</v>
       </c>
       <c r="H78" s="2" t="n">
-        <v>51.84233896740086</v>
+        <v>51.84233896882917</v>
       </c>
       <c r="I78" s="2" t="n">
-        <v>9.63660060987506</v>
+        <v>9.636600611445871</v>
       </c>
       <c r="J78" s="2" t="n">
         <v>0.3769122477709995</v>
@@ -4598,7 +4598,7 @@
         <v>-1</v>
       </c>
       <c r="N78" s="2" t="n">
-        <v>-0.6833467800170778</v>
+        <v>-0.683346779993049</v>
       </c>
       <c r="O78" s="2" t="inlineStr">
         <is>
@@ -4619,7 +4619,7 @@
         <v/>
       </c>
       <c r="D79" s="2" t="n">
-        <v>277.2716068120668</v>
+        <v>277.2716068120662</v>
       </c>
       <c r="E79" s="2" t="n">
         <v>15</v>
@@ -4633,10 +4633,10 @@
         <v>0</v>
       </c>
       <c r="H79" s="2" t="n">
-        <v>48.42739885642819</v>
+        <v>48.42739894551293</v>
       </c>
       <c r="I79" s="2" t="n">
-        <v>11.17146774627873</v>
+        <v>11.17146786423121</v>
       </c>
       <c r="J79" s="2" t="n">
         <v>0.611627332270861</v>
@@ -4686,10 +4686,10 @@
         <v>0</v>
       </c>
       <c r="H80" s="2" t="n">
-        <v>42.06165126115096</v>
+        <v>42.06165113379229</v>
       </c>
       <c r="I80" s="2" t="n">
-        <v>26.62447215558087</v>
+        <v>26.62447214342678</v>
       </c>
       <c r="J80" s="2" t="n">
         <v>0.9096830556558836</v>
@@ -4704,7 +4704,7 @@
         <v>-1</v>
       </c>
       <c r="N80" s="2" t="n">
-        <v>0.0165672795946073</v>
+        <v>0.0165672796787225</v>
       </c>
       <c r="O80" s="2" t="inlineStr">
         <is>
@@ -4739,10 +4739,10 @@
         <v>0</v>
       </c>
       <c r="H81" s="2" t="n">
-        <v>54.33099145935613</v>
+        <v>54.33099149021018</v>
       </c>
       <c r="I81" s="2" t="n">
-        <v>19.41644925304152</v>
+        <v>19.41644931063185</v>
       </c>
       <c r="J81" s="2" t="n">
         <v>0.2335526867460398</v>
@@ -4757,7 +4757,7 @@
         <v>-1</v>
       </c>
       <c r="N81" s="2" t="n">
-        <v>0.0059784922608734</v>
+        <v>0.0059784922488576</v>
       </c>
       <c r="O81" s="2" t="inlineStr">
         <is>
@@ -4792,10 +4792,10 @@
         <v>0</v>
       </c>
       <c r="H82" s="2" t="n">
-        <v>54.69233759732294</v>
+        <v>54.69233756774223</v>
       </c>
       <c r="I82" s="2" t="n">
-        <v>26.29736003015393</v>
+        <v>26.29735998141121</v>
       </c>
       <c r="J82" s="2" t="n">
         <v>0.5449433764223256</v>
@@ -4845,10 +4845,10 @@
         <v>0</v>
       </c>
       <c r="H83" s="2" t="n">
-        <v>39.7877528390004</v>
+        <v>39.78775289530658</v>
       </c>
       <c r="I83" s="2" t="n">
-        <v>7.913383344729607</v>
+        <v>7.913383374352574</v>
       </c>
       <c r="J83" s="2" t="n">
         <v>0.4114168995914857</v>
@@ -4898,10 +4898,10 @@
         <v>0</v>
       </c>
       <c r="H84" s="2" t="n">
-        <v>48.92356581487263</v>
+        <v>48.92356576821288</v>
       </c>
       <c r="I84" s="2" t="n">
-        <v>10.29368007246539</v>
+        <v>10.29368006817163</v>
       </c>
       <c r="J84" s="2" t="n">
         <v>0.1707632648460736</v>
@@ -4916,7 +4916,7 @@
         <v>-1</v>
       </c>
       <c r="N84" s="2" t="n">
-        <v>-0.0308113153727075</v>
+        <v>-0.0308113152525368</v>
       </c>
       <c r="O84" s="2" t="inlineStr">
         <is>
@@ -4951,10 +4951,10 @@
         <v>0</v>
       </c>
       <c r="H85" s="2" t="n">
-        <v>41.25373602648107</v>
+        <v>41.25373583045462</v>
       </c>
       <c r="I85" s="2" t="n">
-        <v>7.022033058927831</v>
+        <v>7.022033024117116</v>
       </c>
       <c r="J85" s="2" t="n">
         <v>0.4968064003889845</v>
@@ -4969,7 +4969,7 @@
         <v>-1</v>
       </c>
       <c r="N85" s="2" t="n">
-        <v>0.09687784268008599</v>
+        <v>0.09687784265604719</v>
       </c>
       <c r="O85" s="2" t="inlineStr">
         <is>
@@ -5004,10 +5004,10 @@
         <v>0</v>
       </c>
       <c r="H86" s="2" t="n">
-        <v>42.56936199569149</v>
+        <v>42.56936194345797</v>
       </c>
       <c r="I86" s="2" t="n">
-        <v>22.82800635326961</v>
+        <v>22.82800637261914</v>
       </c>
       <c r="J86" s="2" t="n">
         <v>0.3666024587756725</v>
@@ -5022,7 +5022,7 @@
         <v>-1</v>
       </c>
       <c r="N86" s="2" t="n">
-        <v>-0.0294667746658545</v>
+        <v>-0.0294667746898886</v>
       </c>
       <c r="O86" s="2" t="inlineStr">
         <is>
@@ -5043,7 +5043,7 @@
         <v/>
       </c>
       <c r="D87" s="2" t="n">
-        <v>257.7244651239454</v>
+        <v>257.7244651239461</v>
       </c>
       <c r="E87" s="2" t="n">
         <v>18.95</v>
@@ -5057,10 +5057,10 @@
         <v>0</v>
       </c>
       <c r="H87" s="2" t="n">
-        <v>21.53347183793444</v>
+        <v>21.53347187246298</v>
       </c>
       <c r="I87" s="2" t="n">
-        <v>43.41795780019862</v>
+        <v>43.41795786373167</v>
       </c>
       <c r="J87" s="2" t="n">
         <v>0.9403330658260024</v>
@@ -5075,7 +5075,7 @@
         <v>-1</v>
       </c>
       <c r="N87" s="2" t="n">
-        <v>-0.0491254250876836</v>
+        <v>-0.0491254251477665</v>
       </c>
       <c r="O87" s="2" t="inlineStr">
         <is>
@@ -5110,10 +5110,10 @@
         <v>0</v>
       </c>
       <c r="H88" s="2" t="n">
-        <v>51.69900279750748</v>
+        <v>51.69900281831584</v>
       </c>
       <c r="I88" s="2" t="n">
-        <v>19.50131410284254</v>
+        <v>19.50131417609135</v>
       </c>
       <c r="J88" s="2" t="n">
         <v>0.4152215415283971</v>
@@ -5128,7 +5128,7 @@
         <v>-1</v>
       </c>
       <c r="N88" s="2" t="n">
-        <v>0.0209995453570373</v>
+        <v>0.0209995453642479</v>
       </c>
       <c r="O88" s="2" t="inlineStr">
         <is>
@@ -5149,7 +5149,7 @@
         <v/>
       </c>
       <c r="D89" s="2" t="n">
-        <v>252.5849449613688</v>
+        <v>252.5849449613692</v>
       </c>
       <c r="E89" s="2" t="n">
         <v>6.13</v>
@@ -5163,10 +5163,10 @@
         <v>0</v>
       </c>
       <c r="H89" s="2" t="n">
-        <v>31.83446723487533</v>
+        <v>31.83446714510077</v>
       </c>
       <c r="I89" s="2" t="n">
-        <v>26.55960084823173</v>
+        <v>26.559600835203</v>
       </c>
       <c r="J89" s="2" t="n">
         <v>0.8111406691347445</v>
@@ -5181,7 +5181,7 @@
         <v>-1</v>
       </c>
       <c r="N89" s="2" t="n">
-        <v>-0.0058522949730176</v>
+        <v>-0.0058522949658073</v>
       </c>
       <c r="O89" s="2" t="inlineStr">
         <is>
@@ -5216,10 +5216,10 @@
         <v>0</v>
       </c>
       <c r="H90" s="2" t="n">
-        <v>51.02451736710853</v>
+        <v>51.0245173489722</v>
       </c>
       <c r="I90" s="2" t="n">
-        <v>19.70385398545727</v>
+        <v>19.70385404808651</v>
       </c>
       <c r="J90" s="2" t="n">
         <v>0.6935591421593238</v>
@@ -5234,7 +5234,7 @@
         <v>-1</v>
       </c>
       <c r="N90" s="2" t="n">
-        <v>0.0271378726032373</v>
+        <v>0.0271378726224656</v>
       </c>
       <c r="O90" s="2" t="inlineStr">
         <is>
@@ -5269,10 +5269,10 @@
         <v>0</v>
       </c>
       <c r="H91" s="2" t="n">
-        <v>37.82205192790969</v>
+        <v>37.82205198441624</v>
       </c>
       <c r="I91" s="2" t="n">
-        <v>25.28069595562538</v>
+        <v>25.28069600926878</v>
       </c>
       <c r="J91" s="2" t="n">
         <v>0.4769121216376146</v>
@@ -5308,7 +5308,7 @@
         <v/>
       </c>
       <c r="D92" s="2" t="n">
-        <v>239.2644748569422</v>
+        <v>239.2644748569421</v>
       </c>
       <c r="E92" s="2" t="n">
         <v>13.35</v>
@@ -5322,10 +5322,10 @@
         <v>0</v>
       </c>
       <c r="H92" s="2" t="n">
-        <v>41.5859457568159</v>
+        <v>41.58594559608561</v>
       </c>
       <c r="I92" s="2" t="n">
-        <v>16.69252899243765</v>
+        <v>16.69252869833998</v>
       </c>
       <c r="J92" s="2" t="n">
         <v>0.330898887024429</v>
@@ -5340,7 +5340,7 @@
         <v>-1</v>
       </c>
       <c r="N92" s="2" t="n">
-        <v>0.0045336953456002</v>
+        <v>0.0045336952734955</v>
       </c>
       <c r="O92" s="2" t="inlineStr">
         <is>
@@ -5375,10 +5375,10 @@
         <v>0</v>
       </c>
       <c r="H93" s="2" t="n">
-        <v>40.26937586414288</v>
+        <v>40.26937577147184</v>
       </c>
       <c r="I93" s="2" t="n">
-        <v>45.48544014622911</v>
+        <v>45.48544006869289</v>
       </c>
       <c r="J93" s="2" t="n">
         <v>0.2675615452417887</v>
@@ -5393,7 +5393,7 @@
         <v>-1</v>
       </c>
       <c r="N93" s="2" t="n">
-        <v>-0.0127954455121749</v>
+        <v>-0.0127954455001571</v>
       </c>
       <c r="O93" s="2" t="inlineStr">
         <is>
@@ -5428,10 +5428,10 @@
         <v>0</v>
       </c>
       <c r="H94" s="2" t="n">
-        <v>47.56717939118548</v>
+        <v>47.56716398570188</v>
       </c>
       <c r="I94" s="2" t="n">
-        <v>6.115329549111436</v>
+        <v>6.115326842474687</v>
       </c>
       <c r="J94" s="2" t="n">
         <v>1.717771848461686</v>
@@ -5446,7 +5446,7 @@
         <v>-1</v>
       </c>
       <c r="N94" s="2" t="n">
-        <v>0.0380618816205615</v>
+        <v>0.0380619917821479</v>
       </c>
       <c r="O94" s="2" t="inlineStr">
         <is>
@@ -5467,7 +5467,7 @@
         <v/>
       </c>
       <c r="D95" s="2" t="n">
-        <v>232.8017503973361</v>
+        <v>232.8017503973362</v>
       </c>
       <c r="E95" s="2" t="n">
         <v>27.8</v>
@@ -5481,10 +5481,10 @@
         <v>0</v>
       </c>
       <c r="H95" s="2" t="n">
-        <v>39.62324749719949</v>
+        <v>39.6232474811784</v>
       </c>
       <c r="I95" s="2" t="n">
-        <v>21.08291409982261</v>
+        <v>21.08291408663561</v>
       </c>
       <c r="J95" s="2" t="n">
         <v>0.5611447521286851</v>
@@ -5499,7 +5499,7 @@
         <v>-1</v>
       </c>
       <c r="N95" s="2" t="n">
-        <v>-0.0235784097678727</v>
+        <v>-0.0235784098039268</v>
       </c>
       <c r="O95" s="2" t="inlineStr">
         <is>
@@ -5520,7 +5520,7 @@
         <v/>
       </c>
       <c r="D96" s="2" t="n">
-        <v>230.6780511349564</v>
+        <v>230.6780511349563</v>
       </c>
       <c r="E96" s="2" t="n">
         <v>13.15</v>
@@ -5537,7 +5537,7 @@
         <v>32.92146106644796</v>
       </c>
       <c r="I96" s="2" t="n">
-        <v>42.59826370699576</v>
+        <v>42.59826373682303</v>
       </c>
       <c r="J96" s="2" t="n">
         <v>0.944552593612224</v>
@@ -5552,7 +5552,7 @@
         <v>-1</v>
       </c>
       <c r="N96" s="2" t="n">
-        <v>-0.0028039409671167</v>
+        <v>-0.0028039409911508</v>
       </c>
       <c r="O96" s="2" t="inlineStr">
         <is>
@@ -5587,10 +5587,10 @@
         <v>0</v>
       </c>
       <c r="H97" s="2" t="n">
-        <v>43.15772217697669</v>
+        <v>43.15772208673069</v>
       </c>
       <c r="I97" s="2" t="n">
-        <v>18.31241188487894</v>
+        <v>18.31241184863592</v>
       </c>
       <c r="J97" s="2" t="n">
         <v>1.01989671559516</v>
@@ -5626,7 +5626,7 @@
         <v/>
       </c>
       <c r="D98" s="2" t="n">
-        <v>229.73830621986</v>
+        <v>229.7383062198601</v>
       </c>
       <c r="E98" s="2" t="n">
         <v>26</v>
@@ -5643,7 +5643,7 @@
         <v>48.00136697318046</v>
       </c>
       <c r="I98" s="2" t="n">
-        <v>19.3791718622256</v>
+        <v>19.3791718720646</v>
       </c>
       <c r="J98" s="2" t="n">
         <v>0.9105529642281216</v>
@@ -5658,7 +5658,7 @@
         <v>-1</v>
       </c>
       <c r="N98" s="2" t="n">
-        <v>-0.0142412689351186</v>
+        <v>-0.0142412687909121</v>
       </c>
       <c r="O98" s="2" t="inlineStr">
         <is>
@@ -5693,10 +5693,10 @@
         <v>0</v>
       </c>
       <c r="H99" s="2" t="n">
-        <v>44.0518392129383</v>
+        <v>44.05183917879359</v>
       </c>
       <c r="I99" s="2" t="n">
-        <v>22.55702016405188</v>
+        <v>22.55702004622144</v>
       </c>
       <c r="J99" s="2" t="n">
         <v>0.6635766342353668</v>
@@ -5746,10 +5746,10 @@
         <v>0</v>
       </c>
       <c r="H100" s="2" t="n">
-        <v>47.51653757506811</v>
+        <v>47.51653748251199</v>
       </c>
       <c r="I100" s="2" t="n">
-        <v>13.48716471547379</v>
+        <v>13.48716472457965</v>
       </c>
       <c r="J100" s="2" t="n">
         <v>0.5194008906363088</v>
@@ -5764,7 +5764,7 @@
         <v>-1</v>
       </c>
       <c r="N100" s="2" t="n">
-        <v>0.009562002489806</v>
+        <v>0.0095620025138375</v>
       </c>
       <c r="O100" s="2" t="inlineStr">
         <is>
@@ -5799,10 +5799,10 @@
         <v>0</v>
       </c>
       <c r="H101" s="2" t="n">
-        <v>43.96490844058936</v>
+        <v>43.96490850801835</v>
       </c>
       <c r="I101" s="2" t="n">
-        <v>11.75004499502716</v>
+        <v>11.7500450680221</v>
       </c>
       <c r="J101" s="2" t="n">
         <v>0.9764873410534992</v>
@@ -5817,7 +5817,7 @@
         <v>-1</v>
       </c>
       <c r="N101" s="2" t="n">
-        <v>-0.6040818310675444</v>
+        <v>-0.6040818334709961</v>
       </c>
       <c r="O101" s="2" t="inlineStr">
         <is>
@@ -5855,7 +5855,7 @@
         <v>43.0442555503309</v>
       </c>
       <c r="I102" s="2" t="n">
-        <v>22.38786703202732</v>
+        <v>22.38786711879305</v>
       </c>
       <c r="J102" s="2" t="n">
         <v>1.205213533985461</v>
@@ -5870,7 +5870,7 @@
         <v>-1</v>
       </c>
       <c r="N102" s="2" t="n">
-        <v>0.0267939333167843</v>
+        <v>0.0267939332927509</v>
       </c>
       <c r="O102" s="2" t="inlineStr">
         <is>
@@ -5905,7 +5905,7 @@
         <v>0</v>
       </c>
       <c r="H103" s="2" t="n">
-        <v>50.01092528761991</v>
+        <v>50.01092533423624</v>
       </c>
       <c r="I103" s="2" t="n">
         <v>10.8164583549112</v>
@@ -5923,7 +5923,7 @@
         <v>-1</v>
       </c>
       <c r="N103" s="2" t="n">
-        <v>-0.0417799901117715</v>
+        <v>-0.0417799902319488</v>
       </c>
       <c r="O103" s="2" t="inlineStr">
         <is>
@@ -5958,10 +5958,10 @@
         <v>0</v>
       </c>
       <c r="H104" s="2" t="n">
-        <v>37.04264004047345</v>
+        <v>37.0426400610569</v>
       </c>
       <c r="I104" s="2" t="n">
-        <v>8.431701713439995</v>
+        <v>8.431701797174629</v>
       </c>
       <c r="J104" s="2" t="n">
         <v>0.5694832965869826</v>
@@ -5976,7 +5976,7 @@
         <v>-1</v>
       </c>
       <c r="N104" s="2" t="n">
-        <v>-0.06391653611123919</v>
+        <v>-0.0639165360992255</v>
       </c>
       <c r="O104" s="2" t="inlineStr">
         <is>
@@ -5997,7 +5997,7 @@
         <v/>
       </c>
       <c r="D105" s="2" t="n">
-        <v>218.4003149853268</v>
+        <v>218.4003149853289</v>
       </c>
       <c r="E105" s="2" t="n">
         <v>26.65</v>
@@ -6011,10 +6011,10 @@
         <v>0</v>
       </c>
       <c r="H105" s="2" t="n">
-        <v>35.33736724989028</v>
+        <v>35.33736728703416</v>
       </c>
       <c r="I105" s="2" t="n">
-        <v>31.64443103445068</v>
+        <v>31.64443087246361</v>
       </c>
       <c r="J105" s="2" t="n">
         <v>0.2389828787257112</v>
@@ -6029,7 +6029,7 @@
         <v>-1</v>
       </c>
       <c r="N105" s="2" t="n">
-        <v>-0.2902966670515259</v>
+        <v>-0.2902966673639767</v>
       </c>
       <c r="O105" s="2" t="inlineStr">
         <is>
@@ -6064,10 +6064,10 @@
         <v>0</v>
       </c>
       <c r="H106" s="2" t="n">
-        <v>51.63874253437996</v>
+        <v>51.63874231922905</v>
       </c>
       <c r="I106" s="2" t="n">
-        <v>11.44358241263085</v>
+        <v>11.44358255590957</v>
       </c>
       <c r="J106" s="2" t="n">
         <v>0.5224568862172136</v>
@@ -6082,7 +6082,7 @@
         <v>-1</v>
       </c>
       <c r="N106" s="2" t="n">
-        <v>0.007026884668629</v>
+        <v>0.007026884788805</v>
       </c>
       <c r="O106" s="2" t="inlineStr">
         <is>
@@ -6117,10 +6117,10 @@
         <v>0</v>
       </c>
       <c r="H107" s="2" t="n">
-        <v>51.14897467808292</v>
+        <v>51.1489746753719</v>
       </c>
       <c r="I107" s="2" t="n">
-        <v>8.117520906096145</v>
+        <v>8.117520810447122</v>
       </c>
       <c r="J107" s="2" t="n">
         <v>0.4576731690936288</v>
@@ -6135,7 +6135,7 @@
         <v>-1</v>
       </c>
       <c r="N107" s="2" t="n">
-        <v>0.3063898763688966</v>
+        <v>0.3063898764049484</v>
       </c>
       <c r="O107" s="2" t="inlineStr">
         <is>
@@ -6156,7 +6156,7 @@
         <v/>
       </c>
       <c r="D108" s="2" t="n">
-        <v>213.9936710765099</v>
+        <v>213.99367107651</v>
       </c>
       <c r="E108" s="2" t="n">
         <v>36</v>
@@ -6170,10 +6170,10 @@
         <v>0</v>
       </c>
       <c r="H108" s="2" t="n">
-        <v>43.36465236607601</v>
+        <v>43.36465244200872</v>
       </c>
       <c r="I108" s="2" t="n">
-        <v>15.39280364553908</v>
+        <v>15.39280372309158</v>
       </c>
       <c r="J108" s="2" t="n">
         <v>0.6149201002736044</v>
@@ -6188,7 +6188,7 @@
         <v>-1</v>
       </c>
       <c r="N108" s="2" t="n">
-        <v>0.0363664547659723</v>
+        <v>0.0363664545736862</v>
       </c>
       <c r="O108" s="2" t="inlineStr">
         <is>
@@ -6223,10 +6223,10 @@
         <v>0</v>
       </c>
       <c r="H109" s="2" t="n">
-        <v>36.35251928457846</v>
+        <v>36.35251915695783</v>
       </c>
       <c r="I109" s="2" t="n">
-        <v>17.29578066225756</v>
+        <v>17.29578073842089</v>
       </c>
       <c r="J109" s="2" t="n">
         <v>1.03227059362489</v>
@@ -6241,7 +6241,7 @@
         <v>-1</v>
       </c>
       <c r="N109" s="2" t="n">
-        <v>0.0009951437709121999</v>
+        <v>0.0009951437829304999</v>
       </c>
       <c r="O109" s="2" t="inlineStr">
         <is>
@@ -6262,7 +6262,7 @@
         <v/>
       </c>
       <c r="D110" s="2" t="n">
-        <v>202.4923153694325</v>
+        <v>202.4923153694324</v>
       </c>
       <c r="E110" s="2" t="n">
         <v>26.4</v>
@@ -6276,10 +6276,10 @@
         <v>0</v>
       </c>
       <c r="H110" s="2" t="n">
-        <v>48.77183447279603</v>
+        <v>48.77183430606079</v>
       </c>
       <c r="I110" s="2" t="n">
-        <v>18.47739421942235</v>
+        <v>18.4773941935249</v>
       </c>
       <c r="J110" s="2" t="n">
         <v>0.8452227454692681</v>
@@ -6294,7 +6294,7 @@
         <v>-1</v>
       </c>
       <c r="N110" s="2" t="n">
-        <v>0.0673968573135123</v>
+        <v>0.0673968572534266</v>
       </c>
       <c r="O110" s="2" t="inlineStr">
         <is>
@@ -6315,7 +6315,7 @@
         <v/>
       </c>
       <c r="D111" s="2" t="n">
-        <v>198.7871125349714</v>
+        <v>198.7871125349721</v>
       </c>
       <c r="E111" s="2" t="n">
         <v>9.880000000000001</v>
@@ -6329,10 +6329,10 @@
         <v>0</v>
       </c>
       <c r="H111" s="2" t="n">
-        <v>40.57251241790832</v>
+        <v>40.57251212911092</v>
       </c>
       <c r="I111" s="2" t="n">
-        <v>16.3562819693102</v>
+        <v>16.35628188281401</v>
       </c>
       <c r="J111" s="2" t="n">
         <v>2.622220555204992</v>
@@ -6347,7 +6347,7 @@
         <v>-1</v>
       </c>
       <c r="N111" s="2" t="n">
-        <v>-0.0063514598265908</v>
+        <v>-0.0063514597785203</v>
       </c>
       <c r="O111" s="2" t="inlineStr">
         <is>
@@ -6368,7 +6368,7 @@
         <v/>
       </c>
       <c r="D112" s="2" t="n">
-        <v>197.7712501278191</v>
+        <v>197.771250127819</v>
       </c>
       <c r="E112" s="2" t="n">
         <v>15.65</v>
@@ -6382,10 +6382,10 @@
         <v>0</v>
       </c>
       <c r="H112" s="2" t="n">
-        <v>44.31756886840401</v>
+        <v>44.31756854502669</v>
       </c>
       <c r="I112" s="2" t="n">
-        <v>18.8686727620981</v>
+        <v>18.86867312423674</v>
       </c>
       <c r="J112" s="2" t="n">
         <v>0.3914240282644893</v>
@@ -6400,7 +6400,7 @@
         <v>-1</v>
       </c>
       <c r="N112" s="2" t="n">
-        <v>0.0855026918930889</v>
+        <v>0.0855026920853663</v>
       </c>
       <c r="O112" s="2" t="inlineStr">
         <is>
@@ -6421,7 +6421,7 @@
         <v/>
       </c>
       <c r="D113" s="2" t="n">
-        <v>193.2078313859375</v>
+        <v>193.2078313859374</v>
       </c>
       <c r="E113" s="2" t="n">
         <v>23.75</v>
@@ -6435,10 +6435,10 @@
         <v>0</v>
       </c>
       <c r="H113" s="2" t="n">
-        <v>37.27863863390674</v>
+        <v>37.27863861312131</v>
       </c>
       <c r="I113" s="2" t="n">
-        <v>6.185853532291535</v>
+        <v>6.18585353483962</v>
       </c>
       <c r="J113" s="2" t="n">
         <v>0.4990335227507368</v>
@@ -6453,7 +6453,7 @@
         <v>-1</v>
       </c>
       <c r="N113" s="2" t="n">
-        <v>0.0034298141110432</v>
+        <v>0.0034298141230608</v>
       </c>
       <c r="O113" s="2" t="inlineStr">
         <is>
@@ -6474,7 +6474,7 @@
         <v/>
       </c>
       <c r="D114" s="2" t="n">
-        <v>186.47221499988</v>
+        <v>186.4722149998801</v>
       </c>
       <c r="E114" s="2" t="n">
         <v>9.31</v>
@@ -6488,10 +6488,10 @@
         <v>0</v>
       </c>
       <c r="H114" s="2" t="n">
-        <v>41.19338205689747</v>
+        <v>41.1933819752071</v>
       </c>
       <c r="I114" s="2" t="n">
-        <v>11.04183603296263</v>
+        <v>11.04183596455273</v>
       </c>
       <c r="J114" s="2" t="n">
         <v>1.063968515593518</v>
@@ -6506,7 +6506,7 @@
         <v>-1</v>
       </c>
       <c r="N114" s="2" t="n">
-        <v>0.0030659955713453</v>
+        <v>0.0030659955953798</v>
       </c>
       <c r="O114" s="2" t="inlineStr">
         <is>
@@ -6541,10 +6541,10 @@
         <v>0</v>
       </c>
       <c r="H115" s="2" t="n">
-        <v>47.54451072648457</v>
+        <v>47.54451076043313</v>
       </c>
       <c r="I115" s="2" t="n">
-        <v>17.48516682565103</v>
+        <v>17.48516654702157</v>
       </c>
       <c r="J115" s="2" t="n">
         <v>0.9005954513582841</v>
@@ -6594,10 +6594,10 @@
         <v>0</v>
       </c>
       <c r="H116" s="2" t="n">
-        <v>39.96530431894045</v>
+        <v>39.96530428444777</v>
       </c>
       <c r="I116" s="2" t="n">
-        <v>14.01694166133939</v>
+        <v>14.01694168685482</v>
       </c>
       <c r="J116" s="2" t="n">
         <v>1.455911996214547</v>
@@ -6612,7 +6612,7 @@
         <v>-1</v>
       </c>
       <c r="N116" s="2" t="n">
-        <v>0.0570931494027361</v>
+        <v>0.0570931494147475</v>
       </c>
       <c r="O116" s="2" t="inlineStr">
         <is>
@@ -6633,7 +6633,7 @@
         <v/>
       </c>
       <c r="D117" s="2" t="n">
-        <v>176.0419416146048</v>
+        <v>176.0419416146047</v>
       </c>
       <c r="E117" s="2" t="n">
         <v>77.90000000000001</v>
@@ -6647,10 +6647,10 @@
         <v>0</v>
       </c>
       <c r="H117" s="2" t="n">
-        <v>31.67443362932927</v>
+        <v>31.67443301054139</v>
       </c>
       <c r="I117" s="2" t="n">
-        <v>16.91842415794158</v>
+        <v>16.91842466422712</v>
       </c>
       <c r="J117" s="2" t="n">
         <v>0.8953143695025576</v>
@@ -6665,7 +6665,7 @@
         <v>-1</v>
       </c>
       <c r="N117" s="2" t="n">
-        <v>-0.0965361360076679</v>
+        <v>-0.0965361354068006</v>
       </c>
       <c r="O117" s="2" t="inlineStr">
         <is>
@@ -6686,7 +6686,7 @@
         <v/>
       </c>
       <c r="D118" s="2" t="n">
-        <v>172.3742163260074</v>
+        <v>172.3742163260075</v>
       </c>
       <c r="E118" s="2" t="n">
         <v>9.949999999999999</v>
@@ -6700,10 +6700,10 @@
         <v>0</v>
       </c>
       <c r="H118" s="2" t="n">
-        <v>51.32341664702017</v>
+        <v>51.32341645358224</v>
       </c>
       <c r="I118" s="2" t="n">
-        <v>15.031989538943</v>
+        <v>15.03198961706072</v>
       </c>
       <c r="J118" s="2" t="n">
         <v>0.8771430071380611</v>
@@ -6718,7 +6718,7 @@
         <v>-1</v>
       </c>
       <c r="N118" s="2" t="n">
-        <v>-0.0049623190631047</v>
+        <v>-0.0049623190510874</v>
       </c>
       <c r="O118" s="2" t="inlineStr">
         <is>
@@ -6739,7 +6739,7 @@
         <v/>
       </c>
       <c r="D119" s="2" t="n">
-        <v>172.2445233747422</v>
+        <v>172.2445233747414</v>
       </c>
       <c r="E119" s="2" t="n">
         <v>106.5</v>
@@ -6756,7 +6756,7 @@
         <v>48.99849359283251</v>
       </c>
       <c r="I119" s="2" t="n">
-        <v>13.91925374940691</v>
+        <v>13.91925379290123</v>
       </c>
       <c r="J119" s="2" t="n">
         <v>0.7911795727396692</v>
@@ -6771,7 +6771,7 @@
         <v>-1</v>
       </c>
       <c r="N119" s="2" t="n">
-        <v>-0.0139062409592394</v>
+        <v>-0.0139062401180267</v>
       </c>
       <c r="O119" s="2" t="inlineStr">
         <is>
@@ -6806,10 +6806,10 @@
         <v>0</v>
       </c>
       <c r="H120" s="2" t="n">
-        <v>44.4906437930235</v>
+        <v>44.49064380210572</v>
       </c>
       <c r="I120" s="2" t="n">
-        <v>9.890374513089109</v>
+        <v>9.890374424151805</v>
       </c>
       <c r="J120" s="2" t="n">
         <v>1.25653611940896</v>
@@ -6824,7 +6824,7 @@
         <v>-1</v>
       </c>
       <c r="N120" s="2" t="n">
-        <v>-0.0119185456445133</v>
+        <v>-0.0119185456324976</v>
       </c>
       <c r="O120" s="2" t="inlineStr">
         <is>
@@ -6859,10 +6859,10 @@
         <v>0</v>
       </c>
       <c r="H121" s="2" t="n">
-        <v>30.40707575332539</v>
+        <v>30.40707570968841</v>
       </c>
       <c r="I121" s="2" t="n">
-        <v>38.55859951359474</v>
+        <v>38.55859948336581</v>
       </c>
       <c r="J121" s="2" t="n">
         <v>0.311157353532924</v>
@@ -6877,7 +6877,7 @@
         <v>-1</v>
       </c>
       <c r="N121" s="2" t="n">
-        <v>-0.0485291746599488</v>
+        <v>-0.0485291746839849</v>
       </c>
       <c r="O121" s="2" t="inlineStr">
         <is>
@@ -6912,10 +6912,10 @@
         <v>0</v>
       </c>
       <c r="H122" s="2" t="n">
-        <v>35.00249362280672</v>
+        <v>35.00249381446193</v>
       </c>
       <c r="I122" s="2" t="n">
-        <v>15.1910321276286</v>
+        <v>15.1910321508628</v>
       </c>
       <c r="J122" s="2" t="n">
         <v>1.237176790090185</v>
@@ -6930,7 +6930,7 @@
         <v>-1</v>
       </c>
       <c r="N122" s="2" t="n">
-        <v>-0.0173587358415028</v>
+        <v>-0.0173587359376394</v>
       </c>
       <c r="O122" s="2" t="inlineStr">
         <is>
@@ -6965,10 +6965,10 @@
         <v>0</v>
       </c>
       <c r="H123" s="2" t="n">
-        <v>49.62774979660142</v>
+        <v>49.62775007002984</v>
       </c>
       <c r="I123" s="2" t="n">
-        <v>13.51074375135028</v>
+        <v>13.5107438868021</v>
       </c>
       <c r="J123" s="2" t="n">
         <v>0.6366568004194362</v>
@@ -6983,7 +6983,7 @@
         <v>-1</v>
       </c>
       <c r="N123" s="2" t="n">
-        <v>0.0280658942830072</v>
+        <v>0.0280658942397453</v>
       </c>
       <c r="O123" s="2" t="inlineStr">
         <is>
@@ -7018,10 +7018,10 @@
         <v>0</v>
       </c>
       <c r="H124" s="2" t="n">
-        <v>51.87251749724368</v>
+        <v>51.87251745258997</v>
       </c>
       <c r="I124" s="2" t="n">
-        <v>12.79069701805218</v>
+        <v>12.79069700624233</v>
       </c>
       <c r="J124" s="2" t="n">
         <v>0.3375353914095136</v>
@@ -7036,7 +7036,7 @@
         <v>-1</v>
       </c>
       <c r="N124" s="2" t="n">
-        <v>0.08222494928221739</v>
+        <v>0.0822249493302861</v>
       </c>
       <c r="O124" s="2" t="inlineStr">
         <is>
@@ -7057,7 +7057,7 @@
         <v/>
       </c>
       <c r="D125" s="2" t="n">
-        <v>155.7147432784423</v>
+        <v>155.7147432784421</v>
       </c>
       <c r="E125" s="2" t="n">
         <v>21.75</v>
@@ -7071,10 +7071,10 @@
         <v>0</v>
       </c>
       <c r="H125" s="2" t="n">
-        <v>35.15927462792179</v>
+        <v>35.15927461270138</v>
       </c>
       <c r="I125" s="2" t="n">
-        <v>20.48553256967309</v>
+        <v>20.48553259193773</v>
       </c>
       <c r="J125" s="2" t="n">
         <v>0.3005727525106256</v>
@@ -7089,7 +7089,7 @@
         <v>-1</v>
       </c>
       <c r="N125" s="2" t="n">
-        <v>-0.0822687415017324</v>
+        <v>-0.0822687415137489</v>
       </c>
       <c r="O125" s="2" t="inlineStr">
         <is>
@@ -7110,7 +7110,7 @@
         <v/>
       </c>
       <c r="D126" s="2" t="n">
-        <v>152.2473752386855</v>
+        <v>152.2473752386857</v>
       </c>
       <c r="E126" s="2" t="n">
         <v>26.2</v>
@@ -7124,10 +7124,10 @@
         <v>0</v>
       </c>
       <c r="H126" s="2" t="n">
-        <v>31.18159486352656</v>
+        <v>31.18159483728992</v>
       </c>
       <c r="I126" s="2" t="n">
-        <v>24.80112969310196</v>
+        <v>24.8011296400756</v>
       </c>
       <c r="J126" s="2" t="n">
         <v>1.025092085012192</v>
@@ -7142,7 +7142,7 @@
         <v>-1</v>
       </c>
       <c r="N126" s="2" t="n">
-        <v>-0.0117486480078891</v>
+        <v>-0.0117486480439383</v>
       </c>
       <c r="O126" s="2" t="inlineStr">
         <is>
@@ -7180,7 +7180,7 @@
         <v>47.39263037244685</v>
       </c>
       <c r="I127" s="2" t="n">
-        <v>8.566954861202273</v>
+        <v>8.566954726772341</v>
       </c>
       <c r="J127" s="2" t="n">
         <v>0.1845698724182319</v>
@@ -7195,7 +7195,7 @@
         <v>-1</v>
       </c>
       <c r="N127" s="2" t="n">
-        <v>0.0391163732146318</v>
+        <v>0.039116373262699</v>
       </c>
       <c r="O127" s="2" t="inlineStr">
         <is>
@@ -7233,7 +7233,7 @@
         <v>51.07066525747229</v>
       </c>
       <c r="I128" s="2" t="n">
-        <v>15.89755363583524</v>
+        <v>15.89755355975165</v>
       </c>
       <c r="J128" s="2" t="n">
         <v>0.6976466133949744</v>
@@ -7248,7 +7248,7 @@
         <v>-1</v>
       </c>
       <c r="N128" s="2" t="n">
-        <v>0.4654882145155766</v>
+        <v>0.4654882145035605</v>
       </c>
       <c r="O128" s="2" t="inlineStr">
         <is>
@@ -7283,10 +7283,10 @@
         <v>0</v>
       </c>
       <c r="H129" s="2" t="n">
-        <v>48.13185912848309</v>
+        <v>48.13185909089826</v>
       </c>
       <c r="I129" s="2" t="n">
-        <v>8.755288046658189</v>
+        <v>8.755288261043026</v>
       </c>
       <c r="J129" s="2" t="n">
         <v>1.101457677301412</v>
@@ -7301,7 +7301,7 @@
         <v>-1</v>
       </c>
       <c r="N129" s="2" t="n">
-        <v>0.0095259637367874</v>
+        <v>0.009525963712752701</v>
       </c>
       <c r="O129" s="2" t="inlineStr">
         <is>
@@ -7336,10 +7336,10 @@
         <v>0</v>
       </c>
       <c r="H130" s="2" t="n">
-        <v>37.95493209600016</v>
+        <v>37.95493172355933</v>
       </c>
       <c r="I130" s="2" t="n">
-        <v>10.84590893064599</v>
+        <v>10.8459089454445</v>
       </c>
       <c r="J130" s="2" t="n">
         <v>0.9647153596768696</v>
@@ -7354,7 +7354,7 @@
         <v>-1</v>
       </c>
       <c r="N130" s="2" t="n">
-        <v>-0.0371663844450914</v>
+        <v>-0.0371663843970234</v>
       </c>
       <c r="O130" s="2" t="inlineStr">
         <is>
@@ -7375,7 +7375,7 @@
         <v/>
       </c>
       <c r="D131" s="2" t="n">
-        <v>82.62113206728273</v>
+        <v>82.62113206728291</v>
       </c>
       <c r="E131" s="2" t="n">
         <v>63.2</v>
@@ -7389,10 +7389,10 @@
         <v>0</v>
       </c>
       <c r="H131" s="2" t="n">
-        <v>50.53786853606798</v>
+        <v>50.53786854367906</v>
       </c>
       <c r="I131" s="2" t="n">
-        <v>13.5747996254918</v>
+        <v>13.57479965575888</v>
       </c>
       <c r="J131" s="2" t="n">
         <v>0.792316615578036</v>
@@ -7407,7 +7407,7 @@
         <v>-1</v>
       </c>
       <c r="N131" s="2" t="n">
-        <v>0.8517572242428235</v>
+        <v>0.8517572240265205</v>
       </c>
       <c r="O131" s="2" t="inlineStr">
         <is>
@@ -7445,7 +7445,7 @@
         <v>44.1707211614111</v>
       </c>
       <c r="I132" s="2" t="n">
-        <v>13.52132577857056</v>
+        <v>13.52132575646312</v>
       </c>
       <c r="J132" s="2" t="n">
         <v>0.5040647235007047</v>
@@ -7460,7 +7460,7 @@
         <v>-1</v>
       </c>
       <c r="N132" s="2" t="n">
-        <v>-0.0231343452758991</v>
+        <v>-0.0231343452999326</v>
       </c>
       <c r="O132" s="2" t="inlineStr">
         <is>
@@ -7481,7 +7481,7 @@
         <v/>
       </c>
       <c r="D133" s="2" t="n">
-        <v>57.7143214625001</v>
+        <v>57.71432146248893</v>
       </c>
       <c r="E133" s="2" t="n">
         <v>12.2</v>
@@ -7495,10 +7495,10 @@
         <v>0</v>
       </c>
       <c r="H133" s="2" t="n">
-        <v>45.35244724899106</v>
+        <v>45.3524472228809</v>
       </c>
       <c r="I133" s="2" t="n">
-        <v>17.19114592414732</v>
+        <v>17.19114604677669</v>
       </c>
       <c r="J133" s="2" t="n">
         <v>1.00129717614731</v>

</xml_diff>